<commit_message>
fix scoridnge code for css
</commit_message>
<xml_diff>
--- a/outputs/pd_css_cross/Gini_vars.xlsx
+++ b/outputs/pd_css_cross/Gini_vars.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="102">
   <si>
     <t>Variable</t>
   </si>
@@ -55,237 +55,258 @@
     <t>Type</t>
   </si>
   <si>
+    <t>act_ccss_min_lninst</t>
+  </si>
+  <si>
+    <t>ags12_Min_CMaxA_Days</t>
+  </si>
+  <si>
+    <t>ags9_Min_CMaxC_Days</t>
+  </si>
+  <si>
+    <t>act12_n_good_days</t>
+  </si>
+  <si>
+    <t>agr12_Mean_CMaxA_Days</t>
+  </si>
+  <si>
     <t>act_ccss_n_statC</t>
   </si>
   <si>
     <t>agr12_Mean_CMaxC_Days</t>
   </si>
   <si>
-    <t>act_ccss_n_loan</t>
-  </si>
-  <si>
-    <t>ags12_Mean_CMaxC_Days</t>
-  </si>
-  <si>
-    <t>agr9_Min_CMaxC_Days</t>
-  </si>
-  <si>
-    <t>agr12_Mean_CMaxA_Days</t>
-  </si>
-  <si>
-    <t>act_ccss_min_lninst</t>
-  </si>
-  <si>
-    <t>ags12_Min_CMaxA_Days</t>
-  </si>
-  <si>
-    <t>ags6_Mean_CMaxA_Days</t>
+    <t>agr6_Mean_CMaxA_Days</t>
+  </si>
+  <si>
+    <t>agr6_Mean_CMaxC_Days</t>
+  </si>
+  <si>
+    <t>ags3_Mean_CMaxA_Days</t>
+  </si>
+  <si>
+    <t>act3_n_good_days</t>
+  </si>
+  <si>
+    <t>act_cins_min_seniority</t>
+  </si>
+  <si>
+    <t>act_ccss_dueutl</t>
   </si>
   <si>
     <t>ags3_Mean_CMaxC_Days</t>
   </si>
   <si>
-    <t>act_ccss_dueutl</t>
+    <t>act_ccss_min_seniority</t>
   </si>
   <si>
     <t>act_ccss_min_pninst</t>
   </si>
   <si>
+    <t>agr6_Mean_CMaxA_Due</t>
+  </si>
+  <si>
+    <t>ags6_Mean_CMaxC_Due</t>
+  </si>
+  <si>
+    <t>act_ccss_cc</t>
+  </si>
+  <si>
+    <t>agr3_Min_CMaxA_Due</t>
+  </si>
+  <si>
+    <t>ags9_Mean_CMaxC_Due</t>
+  </si>
+  <si>
+    <t>ags12_Max_CMaxA_Due</t>
+  </si>
+  <si>
+    <t>ags3_Mean_CMaxC_Due</t>
+  </si>
+  <si>
+    <t>ags12_Min_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>ags12_Mean_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>act_ccss_seniority</t>
+  </si>
+  <si>
+    <t>agr3_Max_CMaxC_Due</t>
+  </si>
+  <si>
+    <t>ags12_Max_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>ags9_Mean_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>ags9_Min_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>ags9_Max_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>agr12_Max_CMaxA_Due</t>
+  </si>
+  <si>
+    <t>ags3_Max_CMaxA_Days</t>
+  </si>
+  <si>
+    <t>ags9_Max_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>ags9_Min_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>ags3_Max_CMaxC_Days</t>
+  </si>
+  <si>
+    <t>agr6_Min_CMaxA_Due</t>
+  </si>
+  <si>
+    <t>ags6_Mean_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>ags6_Mean_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>app_installment</t>
+  </si>
+  <si>
+    <t>ags12_Max_CMaxA_Days</t>
+  </si>
+  <si>
+    <t>ags6_Max_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>act12_n_arrears_days</t>
+  </si>
+  <si>
+    <t>act_cus_active</t>
+  </si>
+  <si>
+    <t>ags12_Min_CMaxA_Due</t>
+  </si>
+  <si>
+    <t>act3_n_arrears_days</t>
+  </si>
+  <si>
+    <t>act_cc</t>
+  </si>
+  <si>
+    <t>agr9_Min_CMaxA_Due</t>
+  </si>
+  <si>
+    <t>act_loaninc</t>
+  </si>
+  <si>
+    <t>ags3_Max_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>ags3_Max_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>act_cins_cc</t>
+  </si>
+  <si>
+    <t>act_cins_min_pninst</t>
+  </si>
+  <si>
     <t>app_number_of_children</t>
   </si>
   <si>
-    <t>act3_n_good_days</t>
-  </si>
-  <si>
-    <t>act_cc</t>
-  </si>
-  <si>
-    <t>agr6_Mean_CMaxA_Due</t>
-  </si>
-  <si>
-    <t>act_ccss_seniority</t>
-  </si>
-  <si>
-    <t>act_ccss_min_seniority</t>
-  </si>
-  <si>
-    <t>act_cins_min_seniority</t>
+    <t>agr12_Min_CMaxA_Due</t>
   </si>
   <si>
     <t>app_income</t>
   </si>
   <si>
-    <t>act_ccss_cc</t>
+    <t>act_cins_utl</t>
   </si>
   <si>
     <t>act_ccss_n_statB</t>
   </si>
   <si>
-    <t>agr9_Max_CMaxC_Due</t>
-  </si>
-  <si>
-    <t>ags12_Max_CMaxI_Due</t>
-  </si>
-  <si>
-    <t>ags12_Min_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>ags12_Mean_CMaxI_Days</t>
+    <t>act_call_cc</t>
+  </si>
+  <si>
+    <t>act_cins_maxdue</t>
+  </si>
+  <si>
+    <t>app_n_installments</t>
+  </si>
+  <si>
+    <t>act_cins_n_loans_act</t>
+  </si>
+  <si>
+    <t>agr6_Max_CMaxA_Days</t>
+  </si>
+  <si>
+    <t>agr6_Mean_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>agr12_Max_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>agr6_Min_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>agr3_Min_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>agr12_Min_CMaxI_Due</t>
+  </si>
+  <si>
+    <t>agr6_Min_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>agr9_Max_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>agr6_Max_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>agr12_Mean_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>agr12_Min_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>act_age</t>
+  </si>
+  <si>
+    <t>agr12_Max_CMaxI_Days</t>
+  </si>
+  <si>
+    <t>act_cins_n_loan</t>
+  </si>
+  <si>
+    <t>app_char_marital_status</t>
   </si>
   <si>
     <t>act_cins_n_statC</t>
   </si>
   <si>
-    <t>ags12_Max_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>ags12_Min_CMaxI_Due</t>
-  </si>
-  <si>
-    <t>ags9_Min_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>ags12_Max_CMaxC_Due</t>
-  </si>
-  <si>
-    <t>agr3_Min_CMaxA_Due</t>
-  </si>
-  <si>
-    <t>ags9_Max_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>app_char_marital_status</t>
-  </si>
-  <si>
-    <t>ags9_Min_CMaxI_Due</t>
-  </si>
-  <si>
-    <t>ags6_Mean_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>ags6_Mean_CMaxI_Due</t>
-  </si>
-  <si>
-    <t>ags6_Max_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>ags3_Max_CMaxC_Days</t>
-  </si>
-  <si>
-    <t>ags6_Min_CMaxI_Due</t>
-  </si>
-  <si>
-    <t>agr6_Max_CMaxC_Days</t>
-  </si>
-  <si>
-    <t>act_cins_min_pninst</t>
-  </si>
-  <si>
-    <t>act_cins_cc</t>
-  </si>
-  <si>
-    <t>ags3_Max_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>act_cins_utl</t>
-  </si>
-  <si>
-    <t>act_age</t>
-  </si>
-  <si>
-    <t>agr12_Max_CMaxI_Due</t>
-  </si>
-  <si>
-    <t>agr9_Min_CMaxI_Due</t>
-  </si>
-  <si>
-    <t>act_cins_maxdue</t>
-  </si>
-  <si>
-    <t>act_cins_n_loans_act</t>
-  </si>
-  <si>
     <t>app_char_gender</t>
   </si>
   <si>
-    <t>agr3_Max_CMaxA_Days</t>
-  </si>
-  <si>
-    <t>agr9_Mean_CMaxI_Days</t>
-  </si>
-  <si>
     <t>app_char_city</t>
   </si>
   <si>
-    <t>ags6_Min_CMaxA_Due</t>
-  </si>
-  <si>
-    <t>act_cins_n_loan</t>
-  </si>
-  <si>
-    <t>agr3_Min_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>agr6_Min_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>agr12_Min_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>agr9_Max_CMaxI_Days</t>
-  </si>
-  <si>
     <t>app_char_home_status</t>
   </si>
   <si>
-    <t>agr6_Max_CMaxI_Days</t>
-  </si>
-  <si>
-    <t>agr12_Max_CMaxI_Days</t>
+    <t>agr9_Max_CMaxC_Days</t>
+  </si>
+  <si>
+    <t>app_char_cars</t>
   </si>
   <si>
     <t>act_cins_n_statB</t>
   </si>
   <si>
-    <t>app_char_cars</t>
-  </si>
-  <si>
-    <t>ags9_Min_CMaxC_Due</t>
-  </si>
-  <si>
-    <t>ags12_Min_CMaxC_Due</t>
-  </si>
-  <si>
-    <t>ags9_Max_CMaxA_Days</t>
-  </si>
-  <si>
-    <t>product</t>
-  </si>
-  <si>
-    <t>ags9_Min_CMaxA_Due</t>
-  </si>
-  <si>
-    <t>act6_n_arrears_days</t>
-  </si>
-  <si>
-    <t>act_cus_active</t>
-  </si>
-  <si>
-    <t>app_char_branch</t>
-  </si>
-  <si>
-    <t>app_installment</t>
-  </si>
-  <si>
-    <t>app_n_installments</t>
-  </si>
-  <si>
-    <t>app_loan_amount</t>
-  </si>
-  <si>
-    <t>ags12_Min_CMaxA_Due</t>
-  </si>
-  <si>
     <t>Maried</t>
   </si>
   <si>
@@ -296,12 +317,6 @@
   </si>
   <si>
     <t>Owner</t>
-  </si>
-  <si>
-    <t>css</t>
-  </si>
-  <si>
-    <t>Empty</t>
   </si>
   <si>
     <t>INT</t>
@@ -662,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -671,7 +686,7 @@
     <col min="5" max="5" width="22.7109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="28.7109375" style="2" customWidth="1"/>
     <col min="7" max="7" width="37.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="20.7109375" style="3" customWidth="1"/>
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="22.7109375" style="1" customWidth="1"/>
@@ -721,37 +736,37 @@
         <v>12</v>
       </c>
       <c r="B2" s="1">
-        <v>0.6662529814075118</v>
+        <v>0.5009587078024258</v>
       </c>
       <c r="C2" s="1">
-        <v>0.6447706281378147</v>
+        <v>0.490353762118569</v>
       </c>
       <c r="D2" s="1">
-        <v>0.03224353791905575</v>
+        <v>0.0211693010195949</v>
       </c>
       <c r="E2" s="2">
-        <v>2.565875312926871</v>
+        <v>0.9276232831164523</v>
       </c>
       <c r="F2" s="2">
-        <v>0.1677511700475778</v>
+        <v>0.02294800237606485</v>
       </c>
       <c r="G2" s="2">
-        <v>0.1936720009617423</v>
+        <v>0.05313321172795519</v>
       </c>
       <c r="H2" s="1">
-        <v>0.0007598784194528875</v>
+        <v>0.3343350864012021</v>
       </c>
       <c r="I2" s="3">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" s="1">
-        <v>0.3707224334600761</v>
+        <v>0.2257336343115124</v>
       </c>
       <c r="L2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -759,37 +774,37 @@
         <v>13</v>
       </c>
       <c r="B3" s="1">
-        <v>0.583720676839373</v>
+        <v>0.4979382762835265</v>
       </c>
       <c r="C3" s="1">
-        <v>0.5320967309240028</v>
+        <v>0.4866588497726427</v>
       </c>
       <c r="D3" s="1">
-        <v>0.08843946764896936</v>
+        <v>0.02265225841859413</v>
       </c>
       <c r="E3" s="2">
-        <v>1.774101651105353</v>
+        <v>0.9211582328635134</v>
       </c>
       <c r="F3" s="2">
-        <v>0.05408817589670517</v>
+        <v>0.01978327431797397</v>
       </c>
       <c r="G3" s="2">
-        <v>0.1018956870132576</v>
+        <v>0.03972923357723279</v>
       </c>
       <c r="H3" s="1">
-        <v>0.3149696048632219</v>
+        <v>0.2566992236413724</v>
       </c>
       <c r="I3" s="3">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="J3">
-        <v>14.83333333333333</v>
+        <v>13</v>
       </c>
       <c r="K3" s="1">
-        <v>0.08707709373266778</v>
+        <v>0.1758760107816712</v>
       </c>
       <c r="L3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -797,37 +812,37 @@
         <v>14</v>
       </c>
       <c r="B4" s="1">
-        <v>0.5711047731256644</v>
+        <v>0.4915181966254489</v>
       </c>
       <c r="C4" s="1">
-        <v>0.5692970017501502</v>
+        <v>0.4810364057539966</v>
       </c>
       <c r="D4" s="1">
-        <v>0.0031653935680143</v>
+        <v>0.02132533636275468</v>
       </c>
       <c r="E4" s="2">
-        <v>1.791625963722091</v>
+        <v>0.9199612715534802</v>
       </c>
       <c r="F4" s="2">
-        <v>0.03458471406023039</v>
+        <v>0.01500221125752964</v>
       </c>
       <c r="G4" s="2">
-        <v>0.08246791661973549</v>
+        <v>0.01297272670509093</v>
       </c>
       <c r="H4" s="1">
-        <v>0</v>
+        <v>0.3265715001252191</v>
       </c>
       <c r="I4" s="3">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="K4" s="1">
-        <v>0.2743161094224924</v>
+        <v>0.171439196727408</v>
       </c>
       <c r="L4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -835,37 +850,37 @@
         <v>15</v>
       </c>
       <c r="B5" s="1">
-        <v>0.5507665450156614</v>
+        <v>0.4840272252938238</v>
       </c>
       <c r="C5" s="1">
-        <v>0.546059607302086</v>
+        <v>0.5013927417279147</v>
       </c>
       <c r="D5" s="1">
-        <v>0.008546157634613569</v>
+        <v>0.03587714807477893</v>
       </c>
       <c r="E5" s="2">
-        <v>1.67977063792685</v>
+        <v>0.8998159700325646</v>
       </c>
       <c r="F5" s="2">
-        <v>0.02689331267147269</v>
+        <v>0.01161177413453514</v>
       </c>
       <c r="G5" s="2">
-        <v>0.05231272733436176</v>
+        <v>0.01696188428399513</v>
       </c>
       <c r="H5" s="1">
-        <v>0.04939209726443769</v>
+        <v>0.2319058352116203</v>
       </c>
       <c r="I5" s="3">
-        <v>157</v>
+        <v>13</v>
       </c>
       <c r="J5">
-        <v>14.83333333333333</v>
+        <v>6</v>
       </c>
       <c r="K5" s="1">
-        <v>0.0627498001598721</v>
+        <v>0.1346592761656342</v>
       </c>
       <c r="L5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -873,37 +888,37 @@
         <v>16</v>
       </c>
       <c r="B6" s="1">
-        <v>0.5440853185436363</v>
+        <v>0.4703001357751102</v>
       </c>
       <c r="C6" s="1">
-        <v>0.4838717919237598</v>
+        <v>0.464323505019018</v>
       </c>
       <c r="D6" s="1">
-        <v>0.1106692729387574</v>
+        <v>0.01270812041387578</v>
       </c>
       <c r="E6" s="2">
-        <v>1.357501082404863</v>
+        <v>0.9006010240118079</v>
       </c>
       <c r="F6" s="2">
-        <v>0.06397359231820764</v>
+        <v>0.006079030319301573</v>
       </c>
       <c r="G6" s="2">
-        <v>0.06554683160843459</v>
+        <v>0.0140370131761075</v>
       </c>
       <c r="H6" s="1">
-        <v>0.2340425531914894</v>
+        <v>0.4019534184823441</v>
       </c>
       <c r="I6" s="3">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="J6">
-        <v>14</v>
+        <v>14.83333333333333</v>
       </c>
       <c r="K6" s="1">
-        <v>0.2058531746031746</v>
+        <v>0.07914572864321608</v>
       </c>
       <c r="L6" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -911,37 +926,37 @@
         <v>17</v>
       </c>
       <c r="B7" s="1">
-        <v>0.5401927258446124</v>
+        <v>0.4213555927549799</v>
       </c>
       <c r="C7" s="1">
-        <v>0.5145824550645766</v>
+        <v>0.4082134584036377</v>
       </c>
       <c r="D7" s="1">
-        <v>0.0474095069310554</v>
+        <v>0.03119012676540992</v>
       </c>
       <c r="E7" s="2">
-        <v>1.420684942501672</v>
+        <v>1.172127812534817</v>
       </c>
       <c r="F7" s="2">
-        <v>0.01644119757498723</v>
+        <v>0.142999048036378</v>
       </c>
       <c r="G7" s="2">
-        <v>0.01651191091593339</v>
+        <v>0.1692973670323071</v>
       </c>
       <c r="H7" s="1">
-        <v>0.1447568389057751</v>
+        <v>0.0843976959679439</v>
       </c>
       <c r="I7" s="3">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="J7">
-        <v>14.83333333333333</v>
+        <v>0</v>
       </c>
       <c r="K7" s="1">
-        <v>0.08085295424255887</v>
+        <v>0.437089715536105</v>
       </c>
       <c r="L7" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -949,37 +964,37 @@
         <v>18</v>
       </c>
       <c r="B8" s="1">
-        <v>0.5358445405519316</v>
+        <v>0.4106388959300094</v>
       </c>
       <c r="C8" s="1">
-        <v>0.4801415449865227</v>
+        <v>0.4512197214516545</v>
       </c>
       <c r="D8" s="1">
-        <v>0.1039536495193804</v>
+        <v>0.09882362806800901</v>
       </c>
       <c r="E8" s="2">
-        <v>1.175084043759764</v>
+        <v>0.8689019265433989</v>
       </c>
       <c r="F8" s="2">
-        <v>0.04975984400324043</v>
+        <v>0.02078944904696788</v>
       </c>
       <c r="G8" s="2">
-        <v>0.08130984785500621</v>
+        <v>0.07963624764651486</v>
       </c>
       <c r="H8" s="1">
-        <v>0.05395136778115502</v>
+        <v>0.5261707988980716</v>
       </c>
       <c r="I8" s="3">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>14.75</v>
       </c>
       <c r="K8" s="1">
-        <v>0.2365461847389558</v>
+        <v>0.08562367864693446</v>
       </c>
       <c r="L8" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -987,37 +1002,37 @@
         <v>19</v>
       </c>
       <c r="B9" s="1">
-        <v>0.5196605266434859</v>
+        <v>0.4050025975460092</v>
       </c>
       <c r="C9" s="1">
-        <v>0.4779442762426704</v>
+        <v>0.3750679211828296</v>
       </c>
       <c r="D9" s="1">
-        <v>0.08027596529269389</v>
+        <v>0.07391230709274388</v>
       </c>
       <c r="E9" s="2">
-        <v>1.145971703676588</v>
+        <v>0.6124917804852319</v>
       </c>
       <c r="F9" s="2">
-        <v>0.01876859097943874</v>
+        <v>0.01611382921776126</v>
       </c>
       <c r="G9" s="2">
-        <v>0.01598421952808288</v>
+        <v>0.01813935017871799</v>
       </c>
       <c r="H9" s="1">
-        <v>0</v>
+        <v>0.3420986726771851</v>
       </c>
       <c r="I9" s="3">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="J9">
-        <v>13</v>
+        <v>14.66666666666667</v>
       </c>
       <c r="K9" s="1">
-        <v>0.1838905775075988</v>
+        <v>0.1191473163304149</v>
       </c>
       <c r="L9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1025,37 +1040,37 @@
         <v>20</v>
       </c>
       <c r="B10" s="1">
-        <v>0.4430712807839305</v>
+        <v>0.3971015402067497</v>
       </c>
       <c r="C10" s="1">
-        <v>0.4040802769580605</v>
+        <v>0.3810106672005034</v>
       </c>
       <c r="D10" s="1">
-        <v>0.08800165011120306</v>
+        <v>0.04052080230630352</v>
       </c>
       <c r="E10" s="2">
-        <v>0.7909477024073525</v>
+        <v>0.6071560284263029</v>
       </c>
       <c r="F10" s="2">
-        <v>0.02447047291241239</v>
+        <v>0.02222943627788453</v>
       </c>
       <c r="G10" s="2">
-        <v>0.0202435222597731</v>
+        <v>0.04369742452719287</v>
       </c>
       <c r="H10" s="1">
-        <v>0</v>
+        <v>0.4227397946406211</v>
       </c>
       <c r="I10" s="3">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="J10">
-        <v>14.66666666666667</v>
+        <v>14.83333333333333</v>
       </c>
       <c r="K10" s="1">
-        <v>0.1109422492401216</v>
+        <v>0.116702819956616</v>
       </c>
       <c r="L10" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1063,37 +1078,37 @@
         <v>21</v>
       </c>
       <c r="B11" s="1">
-        <v>0.4102273053823386</v>
+        <v>0.3921830178214245</v>
       </c>
       <c r="C11" s="1">
-        <v>0.333678253426845</v>
+        <v>0.3648411359281609</v>
       </c>
       <c r="D11" s="1">
-        <v>0.1866015522397971</v>
+        <v>0.06971714901157031</v>
       </c>
       <c r="E11" s="2">
-        <v>0.6171720574508448</v>
+        <v>0.5493465935744124</v>
       </c>
       <c r="F11" s="2">
-        <v>0.04026620343679115</v>
+        <v>0.0203291455745466</v>
       </c>
       <c r="G11" s="2">
-        <v>0.05747437041030902</v>
+        <v>0.03328309279112374</v>
       </c>
       <c r="H11" s="1">
-        <v>0.05357142857142857</v>
+        <v>0.2799899824693213</v>
       </c>
       <c r="I11" s="3">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="J11">
         <v>15</v>
       </c>
       <c r="K11" s="1">
-        <v>0.1770373344038539</v>
+        <v>0.1853913043478261</v>
       </c>
       <c r="L11" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1101,37 +1116,37 @@
         <v>22</v>
       </c>
       <c r="B12" s="1">
-        <v>0.4097316014828012</v>
+        <v>0.389750108544797</v>
       </c>
       <c r="C12" s="1">
-        <v>0.5104945132155496</v>
+        <v>0.3606657705836931</v>
       </c>
       <c r="D12" s="1">
-        <v>0.2459241888301799</v>
+        <v>0.07462304005429415</v>
       </c>
       <c r="E12" s="2">
-        <v>0.7064971482313457</v>
+        <v>0.5288921001635737</v>
       </c>
       <c r="F12" s="2">
-        <v>0.017040882707566</v>
+        <v>0.01976619173023408</v>
       </c>
       <c r="G12" s="2">
-        <v>0.05240989531957951</v>
+        <v>0.02055158504129299</v>
       </c>
       <c r="H12" s="1">
-        <v>0.05395136778115502</v>
+        <v>0.2319058352116203</v>
       </c>
       <c r="I12" s="3">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="J12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K12" s="1">
-        <v>0.5626506024096386</v>
+        <v>0.313009455493968</v>
       </c>
       <c r="L12" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1139,37 +1154,37 @@
         <v>23</v>
       </c>
       <c r="B13" s="1">
-        <v>0.3574935103499144</v>
+        <v>0.3873771812484783</v>
       </c>
       <c r="C13" s="1">
-        <v>0.3485609167209598</v>
+        <v>0.4523293390911429</v>
       </c>
       <c r="D13" s="1">
-        <v>0.02498672946597376</v>
+        <v>0.1676716156417119</v>
       </c>
       <c r="E13" s="2">
-        <v>0.4877115486854892</v>
+        <v>0.5681640141743975</v>
       </c>
       <c r="F13" s="2">
-        <v>0.02944296809588652</v>
+        <v>0.08152339716574526</v>
       </c>
       <c r="G13" s="2">
-        <v>0.0294096935261692</v>
+        <v>0.0624670742334084</v>
       </c>
       <c r="H13" s="1">
-        <v>0.05395136778115502</v>
+        <v>0.02930127723516153</v>
       </c>
       <c r="I13" s="3">
-        <v>25</v>
+        <v>155</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="1">
-        <v>0.3995983935742972</v>
+        <v>0.04437564499484004</v>
       </c>
       <c r="L13" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1177,37 +1192,37 @@
         <v>24</v>
       </c>
       <c r="B14" s="1">
-        <v>0.3464748747569375</v>
+        <v>0.3868960705528632</v>
       </c>
       <c r="C14" s="1">
-        <v>0.3326179435097538</v>
+        <v>0.4558183430091229</v>
       </c>
       <c r="D14" s="1">
-        <v>0.03999404359956759</v>
+        <v>0.1781415674699714</v>
       </c>
       <c r="E14" s="2">
-        <v>0.4974661033575242</v>
+        <v>0.6332338936926084</v>
       </c>
       <c r="F14" s="2">
-        <v>0.05344221626898444</v>
+        <v>0.004948734140416314</v>
       </c>
       <c r="G14" s="2">
-        <v>0.09507281521500392</v>
+        <v>0.02671623249242052</v>
       </c>
       <c r="H14" s="1">
-        <v>0</v>
+        <v>0.3343350864012021</v>
       </c>
       <c r="I14" s="3">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14" s="1">
-        <v>0.4525075987841946</v>
+        <v>0.5628291948833709</v>
       </c>
       <c r="L14" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1215,37 +1230,37 @@
         <v>25</v>
       </c>
       <c r="B15" s="1">
-        <v>0.3332944193798673</v>
+        <v>0.3809583564435455</v>
       </c>
       <c r="C15" s="1">
-        <v>0.2980237356123607</v>
+        <v>0.3084965824920638</v>
       </c>
       <c r="D15" s="1">
-        <v>0.1058244054404862</v>
+        <v>0.1902091730654026</v>
       </c>
       <c r="E15" s="2">
-        <v>0.4192763703945213</v>
+        <v>0.5605303233310432</v>
       </c>
       <c r="F15" s="2">
-        <v>0.01674388034283913</v>
+        <v>0.016999759709203</v>
       </c>
       <c r="G15" s="2">
-        <v>0.0148506172161344</v>
+        <v>0.03498878653147094</v>
       </c>
       <c r="H15" s="1">
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I15" s="3">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="J15">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="K15" s="1">
-        <v>0.3373860182370821</v>
+        <v>0.1754320060105184</v>
       </c>
       <c r="L15" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1253,37 +1268,37 @@
         <v>26</v>
       </c>
       <c r="B16" s="1">
-        <v>0.3271789419236186</v>
+        <v>0.3463417266277329</v>
       </c>
       <c r="C16" s="1">
-        <v>0.338724306646738</v>
+        <v>0.3191237452455173</v>
       </c>
       <c r="D16" s="1">
-        <v>0.03528761556364076</v>
+        <v>0.07858706961829905</v>
       </c>
       <c r="E16" s="2">
-        <v>0.4819709947556169</v>
+        <v>0.4468652465585075</v>
       </c>
       <c r="F16" s="2">
-        <v>0.03934057192931428</v>
+        <v>0.05013097894302458</v>
       </c>
       <c r="G16" s="2">
-        <v>0.06423636558655667</v>
+        <v>0.05839077342539528</v>
       </c>
       <c r="H16" s="1">
-        <v>0</v>
+        <v>0.0843976959679439</v>
       </c>
       <c r="I16" s="3">
-        <v>979</v>
+        <v>123</v>
       </c>
       <c r="J16">
-        <v>0.6056074766355141</v>
+        <v>4</v>
       </c>
       <c r="K16" s="1">
-        <v>0.01063829787234043</v>
+        <v>0.399617067833698</v>
       </c>
       <c r="L16" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1291,37 +1306,37 @@
         <v>27</v>
       </c>
       <c r="B17" s="1">
-        <v>0.3197876854698889</v>
+        <v>0.3387473553969982</v>
       </c>
       <c r="C17" s="1">
-        <v>0.3883289260210274</v>
+        <v>0.3528126519289616</v>
       </c>
       <c r="D17" s="1">
-        <v>0.2143335833911977</v>
+        <v>0.0415214947301344</v>
       </c>
       <c r="E17" s="2">
-        <v>0.3838740655721552</v>
+        <v>0.4508787927830625</v>
       </c>
       <c r="F17" s="2">
-        <v>0.01767080530794175</v>
+        <v>0.01484268367554671</v>
       </c>
       <c r="G17" s="2">
-        <v>0.02910143276005126</v>
+        <v>0.01550058079620635</v>
       </c>
       <c r="H17" s="1">
-        <v>0.0364741641337386</v>
+        <v>0.3343350864012021</v>
       </c>
       <c r="I17" s="3">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="J17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K17" s="1">
-        <v>0.2184542586750789</v>
+        <v>0.3807373965387509</v>
       </c>
       <c r="L17" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1329,37 +1344,37 @@
         <v>28</v>
       </c>
       <c r="B18" s="1">
-        <v>0.3192237324827343</v>
+        <v>0.3374651464539107</v>
       </c>
       <c r="C18" s="1">
-        <v>0.2334342543977312</v>
+        <v>0.3820745274115596</v>
       </c>
       <c r="D18" s="1">
-        <v>0.2687440479997617</v>
+        <v>0.1321895947667633</v>
       </c>
       <c r="E18" s="2">
-        <v>0.4153731686761999</v>
+        <v>0.4389036880092101</v>
       </c>
       <c r="F18" s="2">
-        <v>2.048614522409467</v>
+        <v>0.01214413178640415</v>
       </c>
       <c r="G18" s="2">
-        <v>2.000585500155336</v>
+        <v>0.01915200058008531</v>
       </c>
       <c r="H18" s="1">
-        <v>0.0007598784194528875</v>
+        <v>0.3148009015777611</v>
       </c>
       <c r="I18" s="3">
-        <v>163</v>
+        <v>14</v>
       </c>
       <c r="J18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>0.02053231939163498</v>
+        <v>0.2317251461988304</v>
       </c>
       <c r="L18" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1367,37 +1382,37 @@
         <v>29</v>
       </c>
       <c r="B19" s="1">
-        <v>0.3139505924499748</v>
+        <v>0.335750264146587</v>
       </c>
       <c r="C19" s="1">
-        <v>0.2501692663421862</v>
+        <v>0.4012640489604484</v>
       </c>
       <c r="D19" s="1">
-        <v>0.2031572089418867</v>
+        <v>0.1951265324552608</v>
       </c>
       <c r="E19" s="2">
-        <v>0.3925448239390691</v>
+        <v>0.4152543780407669</v>
       </c>
       <c r="F19" s="2">
-        <v>0.01211809188167572</v>
+        <v>0.006970446485873608</v>
       </c>
       <c r="G19" s="2">
-        <v>0.01826946114433702</v>
+        <v>0.00625408407808732</v>
       </c>
       <c r="H19" s="1">
-        <v>0.0007598784194528875</v>
+        <v>0.3230653643876784</v>
       </c>
       <c r="I19" s="3">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="J19">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K19" s="1">
-        <v>0.5490494296577947</v>
+        <v>0.2253052164261931</v>
       </c>
       <c r="L19" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1405,37 +1420,37 @@
         <v>30</v>
       </c>
       <c r="B20" s="1">
-        <v>0.3076429399312239</v>
+        <v>0.3317392515553907</v>
       </c>
       <c r="C20" s="1">
-        <v>0.3947929840698017</v>
+        <v>0.257396974290045</v>
       </c>
       <c r="D20" s="1">
-        <v>0.2832830948698541</v>
+        <v>0.2240985259259642</v>
       </c>
       <c r="E20" s="2">
-        <v>0.5877038992622926</v>
+        <v>0.3828913371092602</v>
       </c>
       <c r="F20" s="2">
-        <v>0.09708352069240209</v>
+        <v>0.06594841226339736</v>
       </c>
       <c r="G20" s="2">
-        <v>0.03653002855705798</v>
+        <v>0.1065078219537246</v>
       </c>
       <c r="H20" s="1">
-        <v>0</v>
+        <v>0.3343350864012021</v>
       </c>
       <c r="I20" s="3">
-        <v>114</v>
+        <v>1747</v>
       </c>
       <c r="J20">
-        <v>4</v>
+        <v>1.239477503628447</v>
       </c>
       <c r="K20" s="1">
-        <v>0.06306990881458967</v>
+        <v>0.01015801354401806</v>
       </c>
       <c r="L20" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1443,37 +1458,37 @@
         <v>31</v>
       </c>
       <c r="B21" s="1">
-        <v>0.3012508740672626</v>
+        <v>0.3243137835579102</v>
       </c>
       <c r="C21" s="1">
-        <v>0.3644272410224967</v>
+        <v>0.3709440329453484</v>
       </c>
       <c r="D21" s="1">
-        <v>0.2097134727022509</v>
+        <v>0.1437812752695163</v>
       </c>
       <c r="E21" s="2">
-        <v>0.478997712149363</v>
+        <v>0.4148317671352378</v>
       </c>
       <c r="F21" s="2">
-        <v>0.04628106372896016</v>
+        <v>0.0004119193309521045</v>
       </c>
       <c r="G21" s="2">
-        <v>0.08847545004995933</v>
+        <v>0.01221578241462616</v>
       </c>
       <c r="H21" s="1">
-        <v>0</v>
+        <v>0.2857500626095668</v>
       </c>
       <c r="I21" s="3">
-        <v>836</v>
+        <v>3</v>
       </c>
       <c r="J21">
-        <v>1653</v>
+        <v>0</v>
       </c>
       <c r="K21" s="1">
-        <v>0.01253799392097264</v>
+        <v>0.7198457223001402</v>
       </c>
       <c r="L21" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1481,37 +1496,37 @@
         <v>32</v>
       </c>
       <c r="B22" s="1">
-        <v>0.2951647317451651</v>
+        <v>0.3220259353047914</v>
       </c>
       <c r="C22" s="1">
-        <v>0.166379233255407</v>
+        <v>0.3979523550776447</v>
       </c>
       <c r="D22" s="1">
-        <v>0.436317366672882</v>
+        <v>0.2357773441477327</v>
       </c>
       <c r="E22" s="2">
-        <v>0.3457443622258709</v>
+        <v>0.3610480700501807</v>
       </c>
       <c r="F22" s="2">
-        <v>0.1063108829547396</v>
+        <v>0.0118421978802975</v>
       </c>
       <c r="G22" s="2">
-        <v>0.1526660276223776</v>
+        <v>0.003852966558514915</v>
       </c>
       <c r="H22" s="1">
-        <v>0.05395136778115502</v>
+        <v>0.3120460806411219</v>
       </c>
       <c r="I22" s="3">
-        <v>1670</v>
+        <v>66</v>
       </c>
       <c r="J22">
-        <v>1.239477503628447</v>
+        <v>0</v>
       </c>
       <c r="K22" s="1">
-        <v>0.0108433734939759</v>
+        <v>0.1685475063705861</v>
       </c>
       <c r="L22" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1519,37 +1534,37 @@
         <v>33</v>
       </c>
       <c r="B23" s="1">
-        <v>0.2697509267507687</v>
+        <v>0.3206581453772466</v>
       </c>
       <c r="C23" s="1">
-        <v>0.2590477650455421</v>
+        <v>0.3445820344896615</v>
       </c>
       <c r="D23" s="1">
-        <v>0.03967794229346858</v>
+        <v>0.07460870543072924</v>
       </c>
       <c r="E23" s="2">
-        <v>0.3234621213181605</v>
+        <v>0.376426857651166</v>
       </c>
       <c r="F23" s="2">
-        <v>0.08357690389927222</v>
+        <v>0.0284208828603719</v>
       </c>
       <c r="G23" s="2">
-        <v>0.1047267739702687</v>
+        <v>0.03977593401685552</v>
       </c>
       <c r="H23" s="1">
-        <v>0.0007598784194528875</v>
+        <v>0.2434259954921112</v>
       </c>
       <c r="I23" s="3">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="1">
-        <v>0.4806083650190114</v>
+        <v>0.5392254220456802</v>
       </c>
       <c r="L23" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1557,37 +1572,37 @@
         <v>34</v>
       </c>
       <c r="B24" s="1">
-        <v>0.2643442819238098</v>
+        <v>0.3199212956107749</v>
       </c>
       <c r="C24" s="1">
-        <v>0.326383832189987</v>
+        <v>0.3867189063974603</v>
       </c>
       <c r="D24" s="1">
-        <v>0.2346922347427909</v>
+        <v>0.2087938868188171</v>
       </c>
       <c r="E24" s="2">
-        <v>0.2702382453493279</v>
+        <v>0.3838947815943125</v>
       </c>
       <c r="F24" s="2">
-        <v>0.03344660871071819</v>
+        <v>0.01595344691357646</v>
       </c>
       <c r="G24" s="2">
-        <v>0.05213388173552079</v>
+        <v>0.03119582585506425</v>
       </c>
       <c r="H24" s="1">
-        <v>0.1067629179331307</v>
+        <v>0.3283245679939895</v>
       </c>
       <c r="I24" s="3">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="J24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" s="1">
-        <v>0.597618034878775</v>
+        <v>0.3381804623415361</v>
       </c>
       <c r="L24" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1595,37 +1610,37 @@
         <v>35</v>
       </c>
       <c r="B25" s="1">
-        <v>0.2456338544211039</v>
+        <v>0.3048989466762704</v>
       </c>
       <c r="C25" s="1">
-        <v>0.2758083266265539</v>
+        <v>0.2861955558097633</v>
       </c>
       <c r="D25" s="1">
-        <v>0.1228432956709632</v>
+        <v>0.06134291728585601</v>
       </c>
       <c r="E25" s="2">
-        <v>0.2331465062294683</v>
+        <v>0.3500543278598712</v>
       </c>
       <c r="F25" s="2">
-        <v>0.1278064250728748</v>
+        <v>0.04556707276685026</v>
       </c>
       <c r="G25" s="2">
-        <v>0.1066124480960095</v>
+        <v>0.04567795402733907</v>
       </c>
       <c r="H25" s="1">
-        <v>0.3605623100303951</v>
+        <v>0.513648885549712</v>
       </c>
       <c r="I25" s="3">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="J25">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K25" s="1">
-        <v>0.8354129530600118</v>
+        <v>0.1730175077239959</v>
       </c>
       <c r="L25" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1633,37 +1648,37 @@
         <v>36</v>
       </c>
       <c r="B26" s="1">
-        <v>0.2454752052262037</v>
+        <v>0.3037236512210975</v>
       </c>
       <c r="C26" s="1">
-        <v>0.2889408398165538</v>
+        <v>0.2808819744330369</v>
       </c>
       <c r="D26" s="1">
-        <v>0.1770673113412691</v>
+        <v>0.0752054596216903</v>
       </c>
       <c r="E26" s="2">
-        <v>0.2194104907269938</v>
+        <v>0.3628180698467215</v>
       </c>
       <c r="F26" s="2">
-        <v>0.07028758227745933</v>
+        <v>0.0875708582770356</v>
       </c>
       <c r="G26" s="2">
-        <v>0.04251114341530819</v>
+        <v>0.1200443175895783</v>
       </c>
       <c r="H26" s="1">
-        <v>0.3605623100303951</v>
+        <v>0.5128975707488104</v>
       </c>
       <c r="I26" s="3">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="J26">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K26" s="1">
-        <v>0.1740938799762329</v>
+        <v>0.8323907455012853</v>
       </c>
       <c r="L26" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1671,37 +1686,37 @@
         <v>37</v>
       </c>
       <c r="B27" s="1">
-        <v>0.2385856394340833</v>
+        <v>0.3005629271206391</v>
       </c>
       <c r="C27" s="1">
-        <v>0.2894646073659604</v>
+        <v>0.1995824634655532</v>
       </c>
       <c r="D27" s="1">
-        <v>0.2132524323448812</v>
+        <v>0.3359711213304583</v>
       </c>
       <c r="E27" s="2">
-        <v>0.2215145770697367</v>
+        <v>0.3806645360111875</v>
       </c>
       <c r="F27" s="2">
-        <v>0.07673925568057485</v>
+        <v>1.459386074763797</v>
       </c>
       <c r="G27" s="2">
-        <v>0.06251446112612569</v>
+        <v>1.394958320203463</v>
       </c>
       <c r="H27" s="1">
-        <v>0.3605623100303951</v>
+        <v>0.0843976959679439</v>
       </c>
       <c r="I27" s="3">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="J27">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="K27" s="1">
-        <v>0.06833036244800951</v>
+        <v>0.0150437636761488</v>
       </c>
       <c r="L27" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1709,37 +1724,37 @@
         <v>38</v>
       </c>
       <c r="B28" s="1">
-        <v>0.228182442982078</v>
+        <v>0.2951143547670616</v>
       </c>
       <c r="C28" s="1">
-        <v>0.2327955134838207</v>
+        <v>0.3654988989618784</v>
       </c>
       <c r="D28" s="1">
-        <v>0.02021658827671052</v>
+        <v>0.2384992226161699</v>
       </c>
       <c r="E28" s="2">
-        <v>0.1940410927549522</v>
+        <v>0.3271802944170344</v>
       </c>
       <c r="F28" s="2">
-        <v>0.1239140080748635</v>
+        <v>0.01551633398577136</v>
       </c>
       <c r="G28" s="2">
-        <v>0.1039954570281252</v>
+        <v>0.01524403966664175</v>
       </c>
       <c r="H28" s="1">
-        <v>0</v>
+        <v>0.3353368394690709</v>
       </c>
       <c r="I28" s="3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K28" s="1">
-        <v>0.2537993920972644</v>
+        <v>0.5090429540316503</v>
       </c>
       <c r="L28" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1747,37 +1762,37 @@
         <v>39</v>
       </c>
       <c r="B29" s="1">
-        <v>0.2264217362567889</v>
+        <v>0.2925306121424609</v>
       </c>
       <c r="C29" s="1">
-        <v>0.2683861572069137</v>
+        <v>0.280819057968942</v>
       </c>
       <c r="D29" s="1">
-        <v>0.1853374222982386</v>
+        <v>0.04003531147644614</v>
       </c>
       <c r="E29" s="2">
-        <v>0.2113754220475117</v>
+        <v>0.3419020834749247</v>
       </c>
       <c r="F29" s="2">
-        <v>0.06304266416364077</v>
+        <v>0.04114093208484283</v>
       </c>
       <c r="G29" s="2">
-        <v>0.03425842939256065</v>
+        <v>0.02851556832538462</v>
       </c>
       <c r="H29" s="1">
-        <v>0.3605623100303951</v>
+        <v>0.513648885549712</v>
       </c>
       <c r="I29" s="3">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J29">
         <v>15</v>
       </c>
       <c r="K29" s="1">
-        <v>0.8484848484848485</v>
+        <v>0.8486096807415036</v>
       </c>
       <c r="L29" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1785,37 +1800,37 @@
         <v>40</v>
       </c>
       <c r="B30" s="1">
-        <v>0.2188975736850676</v>
+        <v>0.2797777906051655</v>
       </c>
       <c r="C30" s="1">
-        <v>0.2634295277149683</v>
+        <v>0.2602568135670775</v>
       </c>
       <c r="D30" s="1">
-        <v>0.2034374035317987</v>
+        <v>0.06977314745342605</v>
       </c>
       <c r="E30" s="2">
-        <v>0.2075446908183483</v>
+        <v>0.304290128733903</v>
       </c>
       <c r="F30" s="2">
-        <v>0.06273278824942619</v>
+        <v>0.04931476322571716</v>
       </c>
       <c r="G30" s="2">
-        <v>0.03417339251293144</v>
+        <v>0.06100224260785972</v>
       </c>
       <c r="H30" s="1">
-        <v>0.3605623100303951</v>
+        <v>0.5672426746806912</v>
       </c>
       <c r="I30" s="3">
-        <v>4</v>
+        <v>128</v>
       </c>
       <c r="J30">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K30" s="1">
-        <v>0.9910873440285205</v>
+        <v>0.08449074074074074</v>
       </c>
       <c r="L30" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1823,25 +1838,25 @@
         <v>41</v>
       </c>
       <c r="B31" s="1">
-        <v>0.2156012624883856</v>
+        <v>0.2747011567236286</v>
       </c>
       <c r="C31" s="1">
-        <v>0.2657162201867678</v>
+        <v>0.2500643463837333</v>
       </c>
       <c r="D31" s="1">
-        <v>0.2324427840541139</v>
+        <v>0.08968586311663003</v>
       </c>
       <c r="E31" s="2">
-        <v>0.1628840107363335</v>
+        <v>0.2937336497495607</v>
       </c>
       <c r="F31" s="2">
-        <v>0.07456283604647615</v>
+        <v>0.04501355924149052</v>
       </c>
       <c r="G31" s="2">
-        <v>0.04608242314508262</v>
+        <v>0.052463462401166</v>
       </c>
       <c r="H31" s="1">
-        <v>0.4293313069908815</v>
+        <v>0.5672426746806912</v>
       </c>
       <c r="I31" s="3">
         <v>14</v>
@@ -1850,10 +1865,10 @@
         <v>10</v>
       </c>
       <c r="K31" s="1">
-        <v>0.1924101198402131</v>
+        <v>0.1898148148148148</v>
       </c>
       <c r="L31" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1861,37 +1876,37 @@
         <v>42</v>
       </c>
       <c r="B32" s="1">
-        <v>0.2119750807015528</v>
+        <v>0.2715436952413459</v>
       </c>
       <c r="C32" s="1">
-        <v>0.2923900407516704</v>
+        <v>0.2540566820144707</v>
       </c>
       <c r="D32" s="1">
-        <v>0.3793604407837762</v>
+        <v>0.06439852419085945</v>
       </c>
       <c r="E32" s="2">
-        <v>0.1778055739057606</v>
+        <v>0.3003713415493143</v>
       </c>
       <c r="F32" s="2">
-        <v>0.0157250505857816</v>
+        <v>0.08360366196392008</v>
       </c>
       <c r="G32" s="2">
-        <v>0.03323726697429435</v>
+        <v>0.09169562477367502</v>
       </c>
       <c r="H32" s="1">
-        <v>0.0459726443768997</v>
+        <v>0.5657400450788881</v>
       </c>
       <c r="I32" s="3">
         <v>5</v>
       </c>
       <c r="J32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K32" s="1">
-        <v>0.5989645559538033</v>
+        <v>0.8529411764705882</v>
       </c>
       <c r="L32" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1899,37 +1914,37 @@
         <v>43</v>
       </c>
       <c r="B33" s="1">
-        <v>0.2066893684684425</v>
+        <v>0.2681151854798434</v>
       </c>
       <c r="C33" s="1">
-        <v>0.313468490910717</v>
+        <v>0.3213544198816027</v>
       </c>
       <c r="D33" s="1">
-        <v>0.5166164241223544</v>
+        <v>0.1985685156418037</v>
       </c>
       <c r="E33" s="2">
-        <v>0.2266859296241248</v>
+        <v>0.2627781781136743</v>
       </c>
       <c r="F33" s="2">
-        <v>1.361237669762007E-05</v>
+        <v>0.01322707486126032</v>
       </c>
       <c r="G33" s="2">
-        <v>0.01942496024363986</v>
+        <v>0.02124043951109445</v>
       </c>
       <c r="H33" s="1">
-        <v>0</v>
+        <v>0.3453543701477586</v>
       </c>
       <c r="I33" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" s="1">
-        <v>0.712386018237082</v>
+        <v>0.5971690895179801</v>
       </c>
       <c r="L33" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1937,37 +1952,37 @@
         <v>44</v>
       </c>
       <c r="B34" s="1">
-        <v>0.2007528951981379</v>
+        <v>0.265297287258472</v>
       </c>
       <c r="C34" s="1">
-        <v>0.2575786609435482</v>
+        <v>0.2729087425286698</v>
       </c>
       <c r="D34" s="1">
-        <v>0.2830632439413876</v>
+        <v>0.02869028684331085</v>
       </c>
       <c r="E34" s="2">
-        <v>0.1541771283580823</v>
+        <v>0.2942869537048718</v>
       </c>
       <c r="F34" s="2">
-        <v>0.06577590578347758</v>
+        <v>0.001715920351629581</v>
       </c>
       <c r="G34" s="2">
-        <v>0.03773175443746969</v>
+        <v>0.0002609287450701685</v>
       </c>
       <c r="H34" s="1">
-        <v>0.4293313069908815</v>
+        <v>0.2799899824693213</v>
       </c>
       <c r="I34" s="3">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J34">
         <v>15</v>
       </c>
       <c r="K34" s="1">
-        <v>0.822237017310253</v>
+        <v>0.807304347826087</v>
       </c>
       <c r="L34" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1975,37 +1990,37 @@
         <v>45</v>
       </c>
       <c r="B35" s="1">
-        <v>0.1935226826441372</v>
+        <v>0.2620406923777709</v>
       </c>
       <c r="C35" s="1">
-        <v>0.1949054024706498</v>
+        <v>0.2558583807590014</v>
       </c>
       <c r="D35" s="1">
-        <v>0.007145001338449059</v>
+        <v>0.02359294490741483</v>
       </c>
       <c r="E35" s="2">
-        <v>0.1593967340665566</v>
+        <v>0.2821795441014486</v>
       </c>
       <c r="F35" s="2">
-        <v>0.1243833308729017</v>
+        <v>0.04244426382358132</v>
       </c>
       <c r="G35" s="2">
-        <v>0.1581974497963651</v>
+        <v>0.03283561798817289</v>
       </c>
       <c r="H35" s="1">
-        <v>0</v>
+        <v>0.5672426746806912</v>
       </c>
       <c r="I35" s="3">
-        <v>4</v>
-      </c>
-      <c r="J35" t="s">
-        <v>89</v>
+        <v>15</v>
+      </c>
+      <c r="J35">
+        <v>15</v>
       </c>
       <c r="K35" s="1">
-        <v>0.5284954407294833</v>
+        <v>0.8287037037037037</v>
       </c>
       <c r="L35" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2013,37 +2028,37 @@
         <v>46</v>
       </c>
       <c r="B36" s="1">
-        <v>0.1914087569566176</v>
+        <v>0.2598321508433867</v>
       </c>
       <c r="C36" s="1">
-        <v>0.2475887530499878</v>
+        <v>0.2512426001658707</v>
       </c>
       <c r="D36" s="1">
-        <v>0.2935079720835514</v>
+        <v>0.03305807479803884</v>
       </c>
       <c r="E36" s="2">
-        <v>0.1501195532008691</v>
+        <v>0.2822466329238106</v>
       </c>
       <c r="F36" s="2">
-        <v>0.06387209082175055</v>
+        <v>0.04255889692471393</v>
       </c>
       <c r="G36" s="2">
-        <v>0.03017436907932608</v>
+        <v>0.02897888856231333</v>
       </c>
       <c r="H36" s="1">
-        <v>0.4293313069908815</v>
+        <v>0.5657400450788881</v>
       </c>
       <c r="I36" s="3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J36">
         <v>0</v>
       </c>
       <c r="K36" s="1">
-        <v>0.9933422103861518</v>
+        <v>0.9890426758938869</v>
       </c>
       <c r="L36" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2051,37 +2066,37 @@
         <v>47</v>
       </c>
       <c r="B37" s="1">
-        <v>0.1798094054426851</v>
+        <v>0.2502084311073074</v>
       </c>
       <c r="C37" s="1">
-        <v>0.2041926953589086</v>
+        <v>0.2683501587210799</v>
       </c>
       <c r="D37" s="1">
-        <v>0.1356063096710243</v>
+        <v>0.07250646004807108</v>
       </c>
       <c r="E37" s="2">
-        <v>0.1221315614405642</v>
+        <v>0.2536888314697024</v>
       </c>
       <c r="F37" s="2">
-        <v>0.06243047786632831</v>
+        <v>0.01064217228447786</v>
       </c>
       <c r="G37" s="2">
-        <v>0.04945171420172816</v>
+        <v>0.02261480451374505</v>
       </c>
       <c r="H37" s="1">
-        <v>0.5037993920972644</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I37" s="3">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="J37">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K37" s="1">
-        <v>0.08499234303215926</v>
+        <v>0.775732531930879</v>
       </c>
       <c r="L37" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2089,37 +2104,37 @@
         <v>48</v>
       </c>
       <c r="B38" s="1">
-        <v>0.1739070567161891</v>
+        <v>0.2457223311155896</v>
       </c>
       <c r="C38" s="1">
-        <v>0.194062264464288</v>
+        <v>0.2685617868275803</v>
       </c>
       <c r="D38" s="1">
-        <v>0.115896434156732</v>
+        <v>0.09294822985073665</v>
       </c>
       <c r="E38" s="2">
-        <v>0.1343905330746169</v>
+        <v>0.2971374912294183</v>
       </c>
       <c r="F38" s="2">
-        <v>0.07952208175152028</v>
+        <v>0.0001108929109586021</v>
       </c>
       <c r="G38" s="2">
-        <v>0.07175768995707557</v>
+        <v>0.004352947199363634</v>
       </c>
       <c r="H38" s="1">
-        <v>0.5037993920972644</v>
+        <v>0.3148009015777611</v>
       </c>
       <c r="I38" s="3">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="J38">
         <v>0</v>
       </c>
       <c r="K38" s="1">
-        <v>0.8759571209800919</v>
+        <v>0.9031432748538012</v>
       </c>
       <c r="L38" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2127,37 +2142,37 @@
         <v>49</v>
       </c>
       <c r="B39" s="1">
-        <v>0.1691278245543455</v>
+        <v>0.2349203042767904</v>
       </c>
       <c r="C39" s="1">
-        <v>0.198507901225105</v>
+        <v>0.2123945434266594</v>
       </c>
       <c r="D39" s="1">
-        <v>0.1737152165717052</v>
+        <v>0.09588681965774432</v>
       </c>
       <c r="E39" s="2">
-        <v>0.1102345252282423</v>
+        <v>0.2292050814763591</v>
       </c>
       <c r="F39" s="2">
-        <v>0.06143897936273605</v>
+        <v>0.03873353170043941</v>
       </c>
       <c r="G39" s="2">
-        <v>0.04199999289983375</v>
+        <v>0.04321127758000345</v>
       </c>
       <c r="H39" s="1">
-        <v>0.5037993920972644</v>
+        <v>0.6235912847483095</v>
       </c>
       <c r="I39" s="3">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="J39">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K39" s="1">
-        <v>0.7588055130168453</v>
+        <v>0.08383233532934131</v>
       </c>
       <c r="L39" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2165,37 +2180,37 @@
         <v>50</v>
       </c>
       <c r="B40" s="1">
-        <v>0.167849650852036</v>
+        <v>0.2328249504960436</v>
       </c>
       <c r="C40" s="1">
-        <v>0.1370993497617496</v>
+        <v>0.203060028026425</v>
       </c>
       <c r="D40" s="1">
-        <v>0.1832014599624848</v>
+        <v>0.1278424945702905</v>
       </c>
       <c r="E40" s="2">
-        <v>0.1758899494423568</v>
+        <v>0.2437094212730299</v>
       </c>
       <c r="F40" s="2">
-        <v>0.02123272597216982</v>
+        <v>0.05660948236000998</v>
       </c>
       <c r="G40" s="2">
-        <v>0.03556855243356397</v>
+        <v>0.07331271798822771</v>
       </c>
       <c r="H40" s="1">
-        <v>0.05357142857142857</v>
+        <v>0.6225895316804407</v>
       </c>
       <c r="I40" s="3">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="J40">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K40" s="1">
-        <v>0.7796065837013247</v>
+        <v>0.873921698739217</v>
       </c>
       <c r="L40" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2203,37 +2218,37 @@
         <v>51</v>
       </c>
       <c r="B41" s="1">
-        <v>0.1590562947211127</v>
+        <v>0.2286061342241117</v>
       </c>
       <c r="C41" s="1">
-        <v>0.1877004049617395</v>
+        <v>0.2378928704206824</v>
       </c>
       <c r="D41" s="1">
-        <v>0.1800878757477091</v>
+        <v>0.04062330273021705</v>
       </c>
       <c r="E41" s="2">
-        <v>0.1021919398572121</v>
+        <v>0.235145293314636</v>
       </c>
       <c r="F41" s="2">
-        <v>0.04810474666401682</v>
+        <v>0.005463941651158738</v>
       </c>
       <c r="G41" s="2">
-        <v>0.02770766883411296</v>
+        <v>0.01423693824993645</v>
       </c>
       <c r="H41" s="1">
-        <v>0.5037993920972644</v>
+        <v>0</v>
       </c>
       <c r="I41" s="3">
-        <v>2</v>
+        <v>399</v>
       </c>
       <c r="J41">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="K41" s="1">
-        <v>0.9854517611026034</v>
+        <v>0.6609065865264212</v>
       </c>
       <c r="L41" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2241,37 +2256,37 @@
         <v>52</v>
       </c>
       <c r="B42" s="1">
-        <v>0.1583390806249221</v>
+        <v>0.2285898211332329</v>
       </c>
       <c r="C42" s="1">
-        <v>0.117477228886419</v>
+        <v>0.2328252352217803</v>
       </c>
       <c r="D42" s="1">
-        <v>0.2580654856478405</v>
+        <v>0.01852844570047081</v>
       </c>
       <c r="E42" s="2">
-        <v>0.1857870250353962</v>
+        <v>0.2700306921019262</v>
       </c>
       <c r="F42" s="2">
-        <v>0.02404141262804082</v>
+        <v>0.007339999149756883</v>
       </c>
       <c r="G42" s="2">
-        <v>0.02753790350543023</v>
+        <v>0.01136679098636473</v>
       </c>
       <c r="H42" s="1">
-        <v>0.1705927051671733</v>
+        <v>0.2566992236413724</v>
       </c>
       <c r="I42" s="3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="J42">
         <v>15</v>
       </c>
       <c r="K42" s="1">
-        <v>0.9326614750343564</v>
+        <v>0.9228436657681941</v>
       </c>
       <c r="L42" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2279,37 +2294,37 @@
         <v>53</v>
       </c>
       <c r="B43" s="1">
-        <v>0.1564305008764619</v>
+        <v>0.2278303840101592</v>
       </c>
       <c r="C43" s="1">
-        <v>0.1288084926991915</v>
+        <v>0.2070866817284869</v>
       </c>
       <c r="D43" s="1">
-        <v>0.1765768697441199</v>
+        <v>0.09104888433470464</v>
       </c>
       <c r="E43" s="2">
-        <v>0.1190220481301303</v>
+        <v>0.223869406376692</v>
       </c>
       <c r="F43" s="2">
-        <v>0.04481414978646773</v>
+        <v>0.03981030029198934</v>
       </c>
       <c r="G43" s="2">
-        <v>0.03129745880811066</v>
+        <v>0.03406836879934998</v>
       </c>
       <c r="H43" s="1">
-        <v>0.604483282674772</v>
+        <v>0.6235912847483095</v>
       </c>
       <c r="I43" s="3">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="K43" s="1">
-        <v>0.1421709894332373</v>
+        <v>0.761144377910845</v>
       </c>
       <c r="L43" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2317,37 +2332,37 @@
         <v>54</v>
       </c>
       <c r="B44" s="1">
-        <v>0.1488476680364379</v>
+        <v>0.2249705736937608</v>
       </c>
       <c r="C44" s="1">
-        <v>0.1452752334598042</v>
+        <v>0.2233019704292618</v>
       </c>
       <c r="D44" s="1">
-        <v>0.02400060829813717</v>
+        <v>0.007416984528698388</v>
       </c>
       <c r="E44" s="2">
-        <v>0.1435101009045863</v>
+        <v>0.2808302282109769</v>
       </c>
       <c r="F44" s="2">
-        <v>0.1231251664658371</v>
+        <v>0.01499156846789048</v>
       </c>
       <c r="G44" s="2">
-        <v>0.1158157096304569</v>
+        <v>0.021101173556497</v>
       </c>
       <c r="H44" s="1">
-        <v>0.604483282674772</v>
+        <v>0.2319058352116203</v>
       </c>
       <c r="I44" s="3">
-        <v>659</v>
+        <v>5</v>
       </c>
       <c r="J44">
-        <v>0.3035714285714285</v>
+        <v>0</v>
       </c>
       <c r="K44" s="1">
-        <v>0.008645533141210375</v>
+        <v>0.9354417998043691</v>
       </c>
       <c r="L44" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2355,37 +2370,37 @@
         <v>55</v>
       </c>
       <c r="B45" s="1">
-        <v>0.1441809870015422</v>
+        <v>0.2243519310935043</v>
       </c>
       <c r="C45" s="1">
-        <v>0.1542942551642204</v>
+        <v>0.2128349586753226</v>
       </c>
       <c r="D45" s="1">
-        <v>0.07014286954888112</v>
+        <v>0.05133440288232522</v>
       </c>
       <c r="E45" s="2">
-        <v>0.08298097598689448</v>
+        <v>0.2578009918181394</v>
       </c>
       <c r="F45" s="2">
-        <v>0.05278456571431581</v>
+        <v>0.0001440776159210759</v>
       </c>
       <c r="G45" s="2">
-        <v>0.03604323420857695</v>
+        <v>0.0002035800524364324</v>
       </c>
       <c r="H45" s="1">
-        <v>0.5721884498480243</v>
+        <v>0.2824943651389932</v>
       </c>
       <c r="I45" s="3">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="J45">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="K45" s="1">
-        <v>0.5044404973357016</v>
+        <v>1</v>
       </c>
       <c r="L45" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2393,37 +2408,37 @@
         <v>56</v>
       </c>
       <c r="B46" s="1">
-        <v>0.1361832715499487</v>
+        <v>0.2208403500538334</v>
       </c>
       <c r="C46" s="1">
-        <v>0.1242095581190359</v>
+        <v>0.2085280407241112</v>
       </c>
       <c r="D46" s="1">
-        <v>0.0879235261029923</v>
+        <v>0.05575208211144764</v>
       </c>
       <c r="E46" s="2">
-        <v>0.104910864350626</v>
+        <v>0.278904705096408</v>
       </c>
       <c r="F46" s="2">
-        <v>0.04719022499063927</v>
+        <v>0.005946239989673224</v>
       </c>
       <c r="G46" s="2">
-        <v>0.02908252070255192</v>
+        <v>0.004510861051528262</v>
       </c>
       <c r="H46" s="1">
-        <v>0.604483282674772</v>
+        <v>0.2434259954921112</v>
       </c>
       <c r="I46" s="3">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="J46">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="K46" s="1">
-        <v>0.0845341018251681</v>
+        <v>0.9589539887454486</v>
       </c>
       <c r="L46" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2431,37 +2446,37 @@
         <v>57</v>
       </c>
       <c r="B47" s="1">
-        <v>0.1348542103700299</v>
+        <v>0.2163873781851309</v>
       </c>
       <c r="C47" s="1">
-        <v>0.09804673028526167</v>
+        <v>0.2043526753796436</v>
       </c>
       <c r="D47" s="1">
-        <v>0.2729427578402723</v>
+        <v>0.05561647313454168</v>
       </c>
       <c r="E47" s="2">
-        <v>0.08261788630808689</v>
+        <v>0.2779541347488008</v>
       </c>
       <c r="F47" s="2">
-        <v>0.5322184811223956</v>
+        <v>0.009777436546097182</v>
       </c>
       <c r="G47" s="2">
-        <v>0.7893766482389402</v>
+        <v>0.009006523395905786</v>
       </c>
       <c r="H47" s="1">
-        <v>0</v>
+        <v>0.2319058352116203</v>
       </c>
       <c r="I47" s="3">
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="J47">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="K47" s="1">
-        <v>0.04407294832826748</v>
+        <v>0.9748940332572547</v>
       </c>
       <c r="L47" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2469,37 +2484,37 @@
         <v>58</v>
       </c>
       <c r="B48" s="1">
-        <v>0.1300492351312776</v>
+        <v>0.2067285225610047</v>
       </c>
       <c r="C48" s="1">
-        <v>0.1118690836622847</v>
+        <v>0.1588469128035004</v>
       </c>
       <c r="D48" s="1">
-        <v>0.1397943744201272</v>
+        <v>0.2316158852408703</v>
       </c>
       <c r="E48" s="2">
-        <v>0.09177154048545995</v>
+        <v>0.1580880523227999</v>
       </c>
       <c r="F48" s="2">
-        <v>0.07245302578854328</v>
+        <v>0.05527507494177382</v>
       </c>
       <c r="G48" s="2">
-        <v>0.06801595206284214</v>
+        <v>0.04961472592649454</v>
       </c>
       <c r="H48" s="1">
-        <v>0.6990881458966566</v>
+        <v>0</v>
       </c>
       <c r="I48" s="3">
-        <v>4</v>
+        <v>2315</v>
       </c>
       <c r="J48">
-        <v>0</v>
+        <v>0.6056074766355141</v>
       </c>
       <c r="K48" s="1">
-        <v>0.773989898989899</v>
+        <v>0.007012271475081392</v>
       </c>
       <c r="L48" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2507,25 +2522,25 @@
         <v>59</v>
       </c>
       <c r="B49" s="1">
-        <v>0.1276952402846825</v>
+        <v>0.1964994616680009</v>
       </c>
       <c r="C49" s="1">
-        <v>0.117656076342314</v>
+        <v>0.2051419910201047</v>
       </c>
       <c r="D49" s="1">
-        <v>0.07861815303363906</v>
+        <v>0.04398245816421564</v>
       </c>
       <c r="E49" s="2">
-        <v>0.07757010092666559</v>
+        <v>0.1790490236367884</v>
       </c>
       <c r="F49" s="2">
-        <v>0.03751129246661043</v>
+        <v>2.158084367058451E-05</v>
       </c>
       <c r="G49" s="2">
-        <v>0.03020977091101904</v>
+        <v>0.002891443924929315</v>
       </c>
       <c r="H49" s="1">
-        <v>0.6816109422492401</v>
+        <v>0.3268219383921863</v>
       </c>
       <c r="I49" s="3">
         <v>2</v>
@@ -2534,10 +2549,10 @@
         <v>0</v>
       </c>
       <c r="K49" s="1">
-        <v>0.9952267303102625</v>
+        <v>0.9724702380952381</v>
       </c>
       <c r="L49" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2545,37 +2560,37 @@
         <v>60</v>
       </c>
       <c r="B50" s="1">
-        <v>0.1235781440079695</v>
+        <v>0.1957525730763727</v>
       </c>
       <c r="C50" s="1">
-        <v>0.131452880082781</v>
+        <v>0.2504189664540855</v>
       </c>
       <c r="D50" s="1">
-        <v>0.06372272490436209</v>
+        <v>0.2792627065820723</v>
       </c>
       <c r="E50" s="2">
-        <v>0.08960165697728673</v>
+        <v>0.157252317513543</v>
       </c>
       <c r="F50" s="2">
-        <v>0.04852700345501187</v>
+        <v>0.02925558337268852</v>
       </c>
       <c r="G50" s="2">
-        <v>0.03425524965894949</v>
+        <v>0.07215507917986912</v>
       </c>
       <c r="H50" s="1">
-        <v>0.604483282674772</v>
+        <v>0</v>
       </c>
       <c r="I50" s="3">
-        <v>4</v>
+        <v>2190</v>
       </c>
       <c r="J50">
-        <v>0</v>
+        <v>3.024803387779794</v>
       </c>
       <c r="K50" s="1">
-        <v>0.930835734870317</v>
+        <v>0.008264462809917356</v>
       </c>
       <c r="L50" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2583,37 +2598,37 @@
         <v>61</v>
       </c>
       <c r="B51" s="1">
-        <v>0.1207781353870323</v>
+        <v>0.1942896652804722</v>
       </c>
       <c r="C51" s="1">
-        <v>0.1276970835089872</v>
+        <v>0.1676666571338692</v>
       </c>
       <c r="D51" s="1">
-        <v>0.05728642936722966</v>
+        <v>0.1370274024002802</v>
       </c>
       <c r="E51" s="2">
-        <v>0.0642235622017385</v>
+        <v>0.1832532654604554</v>
       </c>
       <c r="F51" s="2">
-        <v>0.07733113850733574</v>
+        <v>0.04344394422138195</v>
       </c>
       <c r="G51" s="2">
-        <v>0.06414446993848207</v>
+        <v>0.04603950982316321</v>
       </c>
       <c r="H51" s="1">
-        <v>0.604483282674772</v>
+        <v>0.6739293764087152</v>
       </c>
       <c r="I51" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" s="1">
-        <v>0.9048991354466859</v>
+        <v>0.8986175115207373</v>
       </c>
       <c r="L51" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2621,37 +2636,37 @@
         <v>62</v>
       </c>
       <c r="B52" s="1">
-        <v>0.1189378047261895</v>
+        <v>0.1907602653261489</v>
       </c>
       <c r="C52" s="1">
-        <v>0.08007256096782012</v>
+        <v>0.1656990877112707</v>
       </c>
       <c r="D52" s="1">
-        <v>0.3267694729009192</v>
+        <v>0.1313752503543138</v>
       </c>
       <c r="E52" s="2">
-        <v>0.09964895925231557</v>
+        <v>0.1690833038835779</v>
       </c>
       <c r="F52" s="2">
-        <v>0.004400766202089534</v>
+        <v>0.03325244427187334</v>
       </c>
       <c r="G52" s="2">
-        <v>0.007182937750045463</v>
+        <v>0.02824803997953897</v>
       </c>
       <c r="H52" s="1">
-        <v>0</v>
+        <v>0.6749311294765841</v>
       </c>
       <c r="I52" s="3">
-        <v>2</v>
-      </c>
-      <c r="J52" t="s">
-        <v>90</v>
+        <v>12</v>
+      </c>
+      <c r="J52">
+        <v>15</v>
       </c>
       <c r="K52" s="1">
-        <v>0.8104103343465046</v>
+        <v>0.5208012326656395</v>
       </c>
       <c r="L52" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2659,37 +2674,37 @@
         <v>63</v>
       </c>
       <c r="B53" s="1">
-        <v>0.116765208770367</v>
+        <v>0.1870501665190123</v>
       </c>
       <c r="C53" s="1">
-        <v>0.1363328606650571</v>
+        <v>0.1549746904223981</v>
       </c>
       <c r="D53" s="1">
-        <v>0.1675811836483956</v>
+        <v>0.171480607013274</v>
       </c>
       <c r="E53" s="2">
-        <v>0.1070828992559062</v>
+        <v>0.1962842035984887</v>
       </c>
       <c r="F53" s="2">
-        <v>0.001880160745821689</v>
+        <v>0.08628922552626657</v>
       </c>
       <c r="G53" s="2">
-        <v>0.00104984541753423</v>
+        <v>0.08785988459430338</v>
       </c>
       <c r="H53" s="1">
-        <v>0.02697568389057751</v>
+        <v>0.6979714500375658</v>
       </c>
       <c r="I53" s="3">
-        <v>14</v>
+        <v>794</v>
       </c>
       <c r="J53">
-        <v>15</v>
+        <v>0.3035714285714285</v>
       </c>
       <c r="K53" s="1">
-        <v>0.818820773135494</v>
+        <v>0.007462686567164179</v>
       </c>
       <c r="L53" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2697,37 +2712,37 @@
         <v>64</v>
       </c>
       <c r="B54" s="1">
-        <v>0.1120075289519813</v>
+        <v>0.1838728783570458</v>
       </c>
       <c r="C54" s="1">
-        <v>0.09095670614085516</v>
+        <v>0.1576915377355792</v>
       </c>
       <c r="D54" s="1">
-        <v>0.1879411411723119</v>
+        <v>0.1423882676738625</v>
       </c>
       <c r="E54" s="2">
-        <v>0.07313002725936127</v>
+        <v>0.1816991428957717</v>
       </c>
       <c r="F54" s="2">
-        <v>0.03343133518494408</v>
+        <v>0.02917810855103957</v>
       </c>
       <c r="G54" s="2">
-        <v>0.02190756198751482</v>
+        <v>0.03067103545920203</v>
       </c>
       <c r="H54" s="1">
-        <v>0.7135258358662614</v>
+        <v>0.6979714500375658</v>
       </c>
       <c r="I54" s="3">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J54">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="K54" s="1">
-        <v>0.07161803713527852</v>
+        <v>0.1260364842454395</v>
       </c>
       <c r="L54" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2735,22 +2750,22 @@
         <v>65</v>
       </c>
       <c r="B55" s="1">
-        <v>0.1042013898866825</v>
+        <v>0.1833084454126332</v>
       </c>
       <c r="C55" s="1">
-        <v>0.1185247639852323</v>
+        <v>0.1473446392312752</v>
       </c>
       <c r="D55" s="1">
-        <v>0.1374585705058852</v>
+        <v>0.1961928491641637</v>
       </c>
       <c r="E55" s="2">
-        <v>0.03667276949689738</v>
+        <v>0.1863834821633018</v>
       </c>
       <c r="F55" s="2">
-        <v>0.02131368977832147</v>
+        <v>0.04507938092315871</v>
       </c>
       <c r="G55" s="2">
-        <v>0.04002349281975784</v>
+        <v>0.04973774190484756</v>
       </c>
       <c r="H55" s="1">
         <v>0</v>
@@ -2758,14 +2773,14 @@
       <c r="I55" s="3">
         <v>4</v>
       </c>
-      <c r="J55" t="s">
-        <v>91</v>
+      <c r="J55">
+        <v>0</v>
       </c>
       <c r="K55" s="1">
-        <v>0.3332066869300912</v>
+        <v>0.5179063360881543</v>
       </c>
       <c r="L55" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2773,37 +2788,37 @@
         <v>66</v>
       </c>
       <c r="B56" s="1">
-        <v>0.1027783365422377</v>
+        <v>0.1831847168925822</v>
       </c>
       <c r="C56" s="1">
-        <v>0.1243373063018178</v>
+        <v>0.1936625961620957</v>
       </c>
       <c r="D56" s="1">
-        <v>0.2097618086153818</v>
+        <v>0.05719843580432324</v>
       </c>
       <c r="E56" s="2">
-        <v>0.1572301775738573</v>
+        <v>0.1507148019625601</v>
       </c>
       <c r="F56" s="2">
-        <v>0.00071421416791651</v>
+        <v>0.0001250019210948577</v>
       </c>
       <c r="G56" s="2">
-        <v>0.005338111748541298</v>
+        <v>0.003507762574762536</v>
       </c>
       <c r="H56" s="1">
-        <v>0</v>
+        <v>0.3453543701477586</v>
       </c>
       <c r="I56" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J56">
         <v>0</v>
       </c>
       <c r="K56" s="1">
-        <v>0.9061550151975684</v>
+        <v>0.9908186687069626</v>
       </c>
       <c r="L56" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2811,37 +2826,37 @@
         <v>67</v>
       </c>
       <c r="B57" s="1">
-        <v>0.0985085778326964</v>
+        <v>0.1812926493212497</v>
       </c>
       <c r="C57" s="1">
-        <v>0.1331519309137827</v>
+        <v>0.203237338061601</v>
       </c>
       <c r="D57" s="1">
-        <v>0.3516785425521363</v>
+        <v>0.1210456619311989</v>
       </c>
       <c r="E57" s="2">
-        <v>0.04431201801966743</v>
+        <v>0.1264120502368338</v>
       </c>
       <c r="F57" s="2">
-        <v>0.02628143864109001</v>
+        <v>0.05342589289122552</v>
       </c>
       <c r="G57" s="2">
-        <v>0.01103906913653764</v>
+        <v>0.07685765290164391</v>
       </c>
       <c r="H57" s="1">
         <v>0</v>
       </c>
       <c r="I57" s="3">
-        <v>4</v>
+        <v>1238</v>
       </c>
       <c r="J57">
-        <v>0</v>
+        <v>1070</v>
       </c>
       <c r="K57" s="1">
-        <v>0.6633738601823708</v>
+        <v>0.009015777610818933</v>
       </c>
       <c r="L57" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2849,37 +2864,37 @@
         <v>68</v>
       </c>
       <c r="B58" s="1">
-        <v>0.09770156230543003</v>
+        <v>0.1784032244706402</v>
       </c>
       <c r="C58" s="1">
-        <v>0.1150244637770028</v>
+        <v>0.1492950496182113</v>
       </c>
       <c r="D58" s="1">
-        <v>0.1773042422537599</v>
+        <v>0.1631594660847581</v>
       </c>
       <c r="E58" s="2">
-        <v>0.03958310546902492</v>
+        <v>0.156802977086275</v>
       </c>
       <c r="F58" s="2">
-        <v>0.07570980913555261</v>
+        <v>0.02779551108671439</v>
       </c>
       <c r="G58" s="2">
-        <v>0.08197715216863485</v>
+        <v>0.02573898454371022</v>
       </c>
       <c r="H58" s="1">
-        <v>0.6242401215805471</v>
+        <v>0.6979714500375658</v>
       </c>
       <c r="I58" s="3">
-        <v>13</v>
+        <v>85</v>
       </c>
       <c r="J58">
-        <v>11</v>
+        <v>0.25</v>
       </c>
       <c r="K58" s="1">
-        <v>0.1708796764408493</v>
+        <v>0.07877280265339967</v>
       </c>
       <c r="L58" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2887,37 +2902,37 @@
         <v>69</v>
       </c>
       <c r="B59" s="1">
-        <v>0.09305583493778546</v>
+        <v>0.1774911972051911</v>
       </c>
       <c r="C59" s="1">
-        <v>0.09835332592393864</v>
+        <v>0.1262390253667744</v>
       </c>
       <c r="D59" s="1">
-        <v>0.05692809042759038</v>
+        <v>0.2887589505589165</v>
       </c>
       <c r="E59" s="2">
-        <v>0.04449821775153249</v>
+        <v>0.1081866851539793</v>
       </c>
       <c r="F59" s="2">
-        <v>0.03202017531824557</v>
+        <v>0.05299753493298862</v>
       </c>
       <c r="G59" s="2">
-        <v>0.02355555383987093</v>
+        <v>0.05649474891984588</v>
       </c>
       <c r="H59" s="1">
-        <v>0.6819908814589666</v>
+        <v>0.0843976959679439</v>
       </c>
       <c r="I59" s="3">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J59">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K59" s="1">
-        <v>0.2043010752688172</v>
+        <v>0.3646061269146608</v>
       </c>
       <c r="L59" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2925,37 +2940,37 @@
         <v>70</v>
       </c>
       <c r="B60" s="1">
-        <v>0.09080002298916634</v>
+        <v>0.1725162064283619</v>
       </c>
       <c r="C60" s="1">
-        <v>0.08350898708465859</v>
+        <v>0.1262275860096662</v>
       </c>
       <c r="D60" s="1">
-        <v>0.08029773192213471</v>
+        <v>0.2683146202726014</v>
       </c>
       <c r="E60" s="2">
-        <v>0.05517077475655036</v>
+        <v>0.1129926985074831</v>
       </c>
       <c r="F60" s="2">
-        <v>0.0327632430297242</v>
+        <v>0.04767911299888341</v>
       </c>
       <c r="G60" s="2">
-        <v>0.0263118036295096</v>
+        <v>0.09795889575175143</v>
       </c>
       <c r="H60" s="1">
-        <v>0.7389817629179332</v>
+        <v>0</v>
       </c>
       <c r="I60" s="3">
-        <v>12</v>
+        <v>3164</v>
       </c>
       <c r="J60">
-        <v>9</v>
+        <v>1.239477503628447</v>
       </c>
       <c r="K60" s="1">
-        <v>0.1950509461426492</v>
+        <v>0.0067618332081142</v>
       </c>
       <c r="L60" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2963,37 +2978,37 @@
         <v>71</v>
       </c>
       <c r="B61" s="1">
-        <v>0.09070782685326217</v>
+        <v>0.1724798156871701</v>
       </c>
       <c r="C61" s="1">
-        <v>0.09699919518644839</v>
+        <v>0.1494609202962793</v>
       </c>
       <c r="D61" s="1">
-        <v>0.06935860500068811</v>
+        <v>0.1334584878768688</v>
       </c>
       <c r="E61" s="2">
-        <v>0.040963929505135</v>
+        <v>0.1631258969802332</v>
       </c>
       <c r="F61" s="2">
-        <v>0.02644619286661154</v>
+        <v>0.03492502754124011</v>
       </c>
       <c r="G61" s="2">
-        <v>0.01714672430414161</v>
+        <v>0.03289444146043753</v>
       </c>
       <c r="H61" s="1">
-        <v>0.7135258358662614</v>
+        <v>0.6979714500375658</v>
       </c>
       <c r="I61" s="3">
         <v>4</v>
       </c>
       <c r="J61">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K61" s="1">
-        <v>0.9137931034482759</v>
+        <v>0.9270315091210614</v>
       </c>
       <c r="L61" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3001,37 +3016,37 @@
         <v>72</v>
       </c>
       <c r="B62" s="1">
-        <v>0.08583340517447824</v>
+        <v>0.1699118842121905</v>
       </c>
       <c r="C62" s="1">
-        <v>0.06481942794363738</v>
+        <v>0.18387622615609</v>
       </c>
       <c r="D62" s="1">
-        <v>0.2448228307862726</v>
+        <v>0.08218578711339851</v>
       </c>
       <c r="E62" s="2">
-        <v>0.05558994271621101</v>
+        <v>0.154762670550653</v>
       </c>
       <c r="F62" s="2">
-        <v>0.02986209844082324</v>
+        <v>0.004859663478316512</v>
       </c>
       <c r="G62" s="2">
-        <v>0.03454771793451713</v>
+        <v>0.02780113414489771</v>
       </c>
       <c r="H62" s="1">
         <v>0</v>
       </c>
       <c r="I62" s="3">
-        <v>2</v>
-      </c>
-      <c r="J62" t="s">
-        <v>92</v>
+        <v>3</v>
+      </c>
+      <c r="J62">
+        <v>24</v>
       </c>
       <c r="K62" s="1">
-        <v>0.8468844984802432</v>
+        <v>0.7485599799649386</v>
       </c>
       <c r="L62" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3039,37 +3054,37 @@
         <v>73</v>
       </c>
       <c r="B63" s="1">
-        <v>0.08161932335220357</v>
+        <v>0.1692902299643873</v>
       </c>
       <c r="C63" s="1">
-        <v>0.09816170364976551</v>
+        <v>0.1473503589098293</v>
       </c>
       <c r="D63" s="1">
-        <v>0.2026772535981252</v>
+        <v>0.129599156780479</v>
       </c>
       <c r="E63" s="2">
-        <v>0.03057621628955921</v>
+        <v>0.1380421729612692</v>
       </c>
       <c r="F63" s="2">
-        <v>0.03479430477204261</v>
+        <v>0.05350823686463348</v>
       </c>
       <c r="G63" s="2">
-        <v>0.01718756578035716</v>
+        <v>0.04767687959662731</v>
       </c>
       <c r="H63" s="1">
-        <v>0.6819908814589666</v>
+        <v>0.6979714500375658</v>
       </c>
       <c r="I63" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J63">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="K63" s="1">
-        <v>0.7980884109916367</v>
+        <v>0.9046434494195689</v>
       </c>
       <c r="L63" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3077,37 +3092,37 @@
         <v>74</v>
       </c>
       <c r="B64" s="1">
-        <v>0.07429092790022707</v>
+        <v>0.1676032053968723</v>
       </c>
       <c r="C64" s="1">
-        <v>0.0839816553609527</v>
+        <v>0.1830697514799668</v>
       </c>
       <c r="D64" s="1">
-        <v>0.1304429455200817</v>
+        <v>0.09228072963444124</v>
       </c>
       <c r="E64" s="2">
-        <v>0.02938520852450613</v>
+        <v>0.1235367442770412</v>
       </c>
       <c r="F64" s="2">
-        <v>0.02386947891559937</v>
+        <v>0.002364667915135467</v>
       </c>
       <c r="G64" s="2">
-        <v>0.01661513930392332</v>
+        <v>0.001236431126518867</v>
       </c>
       <c r="H64" s="1">
-        <v>0.7389817629179332</v>
+        <v>0.3420986726771851</v>
       </c>
       <c r="I64" s="3">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J64">
         <v>15</v>
       </c>
       <c r="K64" s="1">
-        <v>0.9563318777292577</v>
+        <v>0.9368100494861058</v>
       </c>
       <c r="L64" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3115,37 +3130,37 @@
         <v>75</v>
       </c>
       <c r="B65" s="1">
-        <v>0.05404130386888517</v>
+        <v>0.1560706030573242</v>
       </c>
       <c r="C65" s="1">
-        <v>0.07691718085310262</v>
+        <v>0.1487745588697915</v>
       </c>
       <c r="D65" s="1">
-        <v>0.4233035723882388</v>
+        <v>0.04674835647846443</v>
       </c>
       <c r="E65" s="2">
-        <v>0.02564944928620509</v>
+        <v>0.1395035723169025</v>
       </c>
       <c r="F65" s="2">
-        <v>0.003495565911475748</v>
+        <v>0.04029082735541255</v>
       </c>
       <c r="G65" s="2">
-        <v>0.008898628863039899</v>
+        <v>0.04938557589385165</v>
       </c>
       <c r="H65" s="1">
-        <v>0</v>
+        <v>0.7430503380916604</v>
       </c>
       <c r="I65" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J65">
         <v>0</v>
       </c>
       <c r="K65" s="1">
-        <v>0.8620820668693009</v>
+        <v>0.8538011695906432</v>
       </c>
       <c r="L65" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3153,37 +3168,37 @@
         <v>76</v>
       </c>
       <c r="B66" s="1">
-        <v>0.03755615582823246</v>
+        <v>0.1533731707378285</v>
       </c>
       <c r="C66" s="1">
-        <v>0.03157935078373519</v>
+        <v>0.1278176566476963</v>
       </c>
       <c r="D66" s="1">
-        <v>0.159143152771889</v>
+        <v>0.1666231060308198</v>
       </c>
       <c r="E66" s="2">
-        <v>0.01135843145086143</v>
+        <v>0.1489116777187693</v>
       </c>
       <c r="F66" s="2">
-        <v>0.001650696437803148</v>
+        <v>0.05057710489523651</v>
       </c>
       <c r="G66" s="2">
-        <v>0.001809023209017849</v>
+        <v>0.05535277442590077</v>
       </c>
       <c r="H66" s="1">
-        <v>0</v>
+        <v>0.7833708990733784</v>
       </c>
       <c r="I66" s="3">
-        <v>2</v>
-      </c>
-      <c r="J66" t="s">
-        <v>92</v>
+        <v>4</v>
+      </c>
+      <c r="J66">
+        <v>0</v>
       </c>
       <c r="K66" s="1">
-        <v>0.8575227963525835</v>
+        <v>0.7710982658959538</v>
       </c>
       <c r="L66" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3191,37 +3206,37 @@
         <v>77</v>
       </c>
       <c r="B67" s="1">
-        <v>0.03269729973083524</v>
+        <v>0.1514286503050548</v>
       </c>
       <c r="C67" s="1">
-        <v>0.01177838245250973</v>
+        <v>0.1480595990505333</v>
       </c>
       <c r="D67" s="1">
-        <v>0.639775071658223</v>
+        <v>0.02224844009198046</v>
       </c>
       <c r="E67" s="2">
-        <v>0.02518739124965104</v>
+        <v>0.1233907292757356</v>
       </c>
       <c r="F67" s="2">
-        <v>0.007701741131063212</v>
+        <v>0.02833373846625874</v>
       </c>
       <c r="G67" s="2">
-        <v>0.01318825271676188</v>
+        <v>0.0171248862527999</v>
       </c>
       <c r="H67" s="1">
-        <v>0.04939209726443769</v>
+        <v>0.7430503380916604</v>
       </c>
       <c r="I67" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J67">
         <v>0</v>
       </c>
       <c r="K67" s="1">
-        <v>0.9744204636290967</v>
+        <v>0.98635477582846</v>
       </c>
       <c r="L67" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3229,37 +3244,37 @@
         <v>78</v>
       </c>
       <c r="B68" s="1">
-        <v>0.03009425558205692</v>
+        <v>0.1496505233992467</v>
       </c>
       <c r="C68" s="1">
-        <v>0.01177838245250973</v>
+        <v>0.1472359653387481</v>
       </c>
       <c r="D68" s="1">
-        <v>0.6086169195847347</v>
+        <v>0.01613464494244978</v>
       </c>
       <c r="E68" s="2">
-        <v>0.02280593886292052</v>
+        <v>0.1095142603103395</v>
       </c>
       <c r="F68" s="2">
-        <v>0.005135186633395065</v>
+        <v>0.05280068487957493</v>
       </c>
       <c r="G68" s="2">
-        <v>0.009208642367301498</v>
+        <v>0.06597459595437527</v>
       </c>
       <c r="H68" s="1">
-        <v>0.0459726443768997</v>
+        <v>0.7172551965940396</v>
       </c>
       <c r="I68" s="3">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="J68">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K68" s="1">
-        <v>0.9884508164078056</v>
+        <v>0.1762621789193977</v>
       </c>
       <c r="L68" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3267,37 +3282,37 @@
         <v>79</v>
       </c>
       <c r="B69" s="1">
-        <v>0.01550092435606376</v>
+        <v>0.1494768517240428</v>
       </c>
       <c r="C69" s="1">
-        <v>0.03674037736813207</v>
+        <v>0.1265364486515856</v>
       </c>
       <c r="D69" s="1">
-        <v>1.370205577692514</v>
+        <v>0.1534712753705079</v>
       </c>
       <c r="E69" s="2">
-        <v>0.004757196602893884</v>
+        <v>0.1368353932648988</v>
       </c>
       <c r="F69" s="2">
-        <v>0.008913975280117687</v>
+        <v>0.02722673792644682</v>
       </c>
       <c r="G69" s="2">
-        <v>0.0169583465302509</v>
+        <v>0.02237893100941589</v>
       </c>
       <c r="H69" s="1">
-        <v>0</v>
+        <v>0.7833708990733784</v>
       </c>
       <c r="I69" s="3">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J69">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K69" s="1">
-        <v>0.9395896656534954</v>
+        <v>0.9953757225433526</v>
       </c>
       <c r="L69" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3305,37 +3320,37 @@
         <v>80</v>
       </c>
       <c r="B70" s="1">
-        <v>0</v>
+        <v>0.1310056644070945</v>
       </c>
       <c r="C70" s="1">
-        <v>0</v>
+        <v>0.1328910115251523</v>
       </c>
       <c r="D70" s="1">
-        <v>0</v>
+        <v>0.01439134045531903</v>
       </c>
       <c r="E70" s="2">
-        <v>0</v>
+        <v>0.09824545640079942</v>
       </c>
       <c r="F70" s="2">
-        <v>0</v>
+        <v>0.03277770631091859</v>
       </c>
       <c r="G70" s="2">
-        <v>0</v>
+        <v>0.0442654590793902</v>
       </c>
       <c r="H70" s="1">
-        <v>0</v>
+        <v>0.7615827698472326</v>
       </c>
       <c r="I70" s="3">
-        <v>1</v>
-      </c>
-      <c r="J70" t="s">
-        <v>93</v>
+        <v>14</v>
+      </c>
+      <c r="J70">
+        <v>10</v>
       </c>
       <c r="K70" s="1">
-        <v>1</v>
+        <v>0.2048319327731092</v>
       </c>
       <c r="L70" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3343,37 +3358,37 @@
         <v>81</v>
       </c>
       <c r="B71" s="1">
-        <v>0</v>
+        <v>0.127768896206077</v>
       </c>
       <c r="C71" s="1">
-        <v>0</v>
+        <v>0.1229273314839705</v>
       </c>
       <c r="D71" s="1">
-        <v>0</v>
+        <v>0.03789314039543396</v>
       </c>
       <c r="E71" s="2">
-        <v>0</v>
+        <v>0.1001817016979651</v>
       </c>
       <c r="F71" s="2">
-        <v>0</v>
+        <v>0.02072340165977058</v>
       </c>
       <c r="G71" s="2">
-        <v>0</v>
+        <v>0.0122545491705767</v>
       </c>
       <c r="H71" s="1">
-        <v>0</v>
+        <v>0.7876283496118207</v>
       </c>
       <c r="I71" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J71">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K71" s="1">
-        <v>0.9745440729483282</v>
+        <v>0.9186320754716981</v>
       </c>
       <c r="L71" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3381,37 +3396,37 @@
         <v>82</v>
       </c>
       <c r="B72" s="1">
-        <v>0</v>
+        <v>0.1267341443030923</v>
       </c>
       <c r="C72" s="1">
-        <v>0</v>
+        <v>0.1284639803243057</v>
       </c>
       <c r="D72" s="1">
-        <v>0</v>
+        <v>0.01364932892178176</v>
       </c>
       <c r="E72" s="2">
-        <v>0</v>
+        <v>0.08954797152487119</v>
       </c>
       <c r="F72" s="2">
-        <v>0</v>
+        <v>0.02691936770132914</v>
       </c>
       <c r="G72" s="2">
-        <v>0</v>
+        <v>0.01195262497510266</v>
       </c>
       <c r="H72" s="1">
-        <v>0</v>
+        <v>0.7615827698472326</v>
       </c>
       <c r="I72" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J72">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K72" s="1">
-        <v>0.9578267477203647</v>
+        <v>0.7993697478991597</v>
       </c>
       <c r="L72" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3419,37 +3434,37 @@
         <v>83</v>
       </c>
       <c r="B73" s="1">
-        <v>0</v>
+        <v>0.1141324070843988</v>
       </c>
       <c r="C73" s="1">
-        <v>0</v>
+        <v>0.1083650298853205</v>
       </c>
       <c r="D73" s="1">
-        <v>0</v>
+        <v>0.05053233648891156</v>
       </c>
       <c r="E73" s="2">
-        <v>0</v>
+        <v>0.1130462096906638</v>
       </c>
       <c r="F73" s="2">
-        <v>0</v>
+        <v>0.02142940512989022</v>
       </c>
       <c r="G73" s="2">
-        <v>0</v>
+        <v>0.02510189907468453</v>
       </c>
       <c r="H73" s="1">
-        <v>0</v>
+        <v>0.8126721763085399</v>
       </c>
       <c r="I73" s="3">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="J73">
-        <v>1</v>
+        <v>12.41666666666667</v>
       </c>
       <c r="K73" s="1">
-        <v>1</v>
+        <v>0.05614973262032086</v>
       </c>
       <c r="L73" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3457,37 +3472,37 @@
         <v>84</v>
       </c>
       <c r="B74" s="1">
-        <v>0</v>
+        <v>0.1122531390151411</v>
       </c>
       <c r="C74" s="1">
-        <v>0</v>
+        <v>0.1119913060885978</v>
       </c>
       <c r="D74" s="1">
-        <v>0</v>
+        <v>0.002332522091057449</v>
       </c>
       <c r="E74" s="2">
-        <v>0</v>
+        <v>0.09630938667483455</v>
       </c>
       <c r="F74" s="2">
-        <v>0</v>
+        <v>0.02325605958614658</v>
       </c>
       <c r="G74" s="2">
-        <v>0</v>
+        <v>0.02101695018413658</v>
       </c>
       <c r="H74" s="1">
-        <v>0</v>
+        <v>0.8126721763085399</v>
       </c>
       <c r="I74" s="3">
-        <v>1</v>
-      </c>
-      <c r="J74" t="s">
-        <v>94</v>
+        <v>12</v>
+      </c>
+      <c r="J74">
+        <v>10</v>
       </c>
       <c r="K74" s="1">
-        <v>1</v>
+        <v>0.1978609625668449</v>
       </c>
       <c r="L74" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3495,37 +3510,37 @@
         <v>85</v>
       </c>
       <c r="B75" s="1">
-        <v>0</v>
+        <v>0.1121266498181717</v>
       </c>
       <c r="C75" s="1">
-        <v>0</v>
+        <v>0.04281751365573272</v>
       </c>
       <c r="D75" s="1">
-        <v>0</v>
+        <v>0.6181325873450511</v>
       </c>
       <c r="E75" s="2">
-        <v>0</v>
+        <v>0.04725941257947438</v>
       </c>
       <c r="F75" s="2">
-        <v>0</v>
+        <v>0.3748879554935821</v>
       </c>
       <c r="G75" s="2">
-        <v>0</v>
+        <v>0.2560544596879363</v>
       </c>
       <c r="H75" s="1">
         <v>0</v>
       </c>
       <c r="I75" s="3">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="J75">
-        <v>208</v>
+        <v>64</v>
       </c>
       <c r="K75" s="1">
-        <v>1</v>
+        <v>0.04232406711745555</v>
       </c>
       <c r="L75" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3533,37 +3548,37 @@
         <v>86</v>
       </c>
       <c r="B76" s="1">
-        <v>0</v>
+        <v>0.1072176643167451</v>
       </c>
       <c r="C76" s="1">
-        <v>0</v>
+        <v>0.1084622644207396</v>
       </c>
       <c r="D76" s="1">
-        <v>0</v>
+        <v>0.01160816281464304</v>
       </c>
       <c r="E76" s="2">
-        <v>0</v>
+        <v>0.0774601824242348</v>
       </c>
       <c r="F76" s="2">
-        <v>0</v>
+        <v>0.01583307893132292</v>
       </c>
       <c r="G76" s="2">
-        <v>0</v>
+        <v>0.009287832678639323</v>
       </c>
       <c r="H76" s="1">
-        <v>0</v>
+        <v>0.8126721763085399</v>
       </c>
       <c r="I76" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J76">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="K76" s="1">
-        <v>1</v>
+        <v>0.9585561497326203</v>
       </c>
       <c r="L76" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3571,37 +3586,37 @@
         <v>87</v>
       </c>
       <c r="B77" s="1">
-        <v>0</v>
+        <v>0.09474668279571241</v>
       </c>
       <c r="C77" s="1">
-        <v>0</v>
+        <v>0.08401063860211044</v>
       </c>
       <c r="D77" s="1">
-        <v>0</v>
+        <v>0.1133131406484218</v>
       </c>
       <c r="E77" s="2">
-        <v>0</v>
+        <v>0.0349744298233252</v>
       </c>
       <c r="F77" s="2">
-        <v>0</v>
+        <v>0.02218936553164815</v>
       </c>
       <c r="G77" s="2">
-        <v>0</v>
+        <v>0.03206254865431231</v>
       </c>
       <c r="H77" s="1">
         <v>0</v>
       </c>
       <c r="I77" s="3">
+        <v>5</v>
+      </c>
+      <c r="J77">
         <v>1</v>
       </c>
-      <c r="J77">
-        <v>5000</v>
-      </c>
       <c r="K77" s="1">
-        <v>1</v>
+        <v>0.5036313548710243</v>
       </c>
       <c r="L77" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3609,41 +3624,307 @@
         <v>88</v>
       </c>
       <c r="B78" s="1">
-        <v>0</v>
+        <v>0.09468670081540376</v>
       </c>
       <c r="C78" s="1">
-        <v>0</v>
+        <v>0.1408928418222897</v>
       </c>
       <c r="D78" s="1">
-        <v>0</v>
+        <v>0.4879897663449801</v>
       </c>
       <c r="E78" s="2">
-        <v>0</v>
+        <v>0.03490769983211704</v>
       </c>
       <c r="F78" s="2">
-        <v>0</v>
+        <v>0.1000389537311405</v>
       </c>
       <c r="G78" s="2">
-        <v>0</v>
+        <v>0.1078087772858352</v>
       </c>
       <c r="H78" s="1">
         <v>0</v>
       </c>
       <c r="I78" s="3">
+        <v>4</v>
+      </c>
+      <c r="J78" t="s">
+        <v>96</v>
+      </c>
+      <c r="K78" s="1">
+        <v>0.518908089156023</v>
+      </c>
+      <c r="L78" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12">
+      <c r="A79" t="s">
+        <v>89</v>
+      </c>
+      <c r="B79" s="1">
+        <v>0.08970518480222256</v>
+      </c>
+      <c r="C79" s="1">
+        <v>0.04006062859267323</v>
+      </c>
+      <c r="D79" s="1">
+        <v>0.5534190283315633</v>
+      </c>
+      <c r="E79" s="2">
+        <v>0.02742740396428815</v>
+      </c>
+      <c r="F79" s="2">
+        <v>0.08494612360859065</v>
+      </c>
+      <c r="G79" s="2">
+        <v>0.1039714241579996</v>
+      </c>
+      <c r="H79" s="1">
+        <v>0.02930127723516153</v>
+      </c>
+      <c r="I79" s="3">
+        <v>13</v>
+      </c>
+      <c r="J79">
+        <v>1</v>
+      </c>
+      <c r="K79" s="1">
+        <v>0.2649638802889577</v>
+      </c>
+      <c r="L79" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12">
+      <c r="A80" t="s">
+        <v>90</v>
+      </c>
+      <c r="B80" s="1">
+        <v>0.0636501670209535</v>
+      </c>
+      <c r="C80" s="1">
+        <v>0.01550032888151676</v>
+      </c>
+      <c r="D80" s="1">
+        <v>0.7564762261124298</v>
+      </c>
+      <c r="E80" s="2">
+        <v>0.02375097170521714</v>
+      </c>
+      <c r="F80" s="2">
+        <v>0.003405696122365031</v>
+      </c>
+      <c r="G80" s="2">
+        <v>0.01209125800229851</v>
+      </c>
+      <c r="H80" s="1">
+        <v>0</v>
+      </c>
+      <c r="I80" s="3">
         <v>2</v>
       </c>
-      <c r="J78">
-        <v>0</v>
-      </c>
-      <c r="K78" s="1">
-        <v>0.9916413373860182</v>
-      </c>
-      <c r="L78" t="s">
+      <c r="J80" t="s">
+        <v>97</v>
+      </c>
+      <c r="K80" s="1">
+        <v>0.7796143250688705</v>
+      </c>
+      <c r="L80" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12">
+      <c r="A81" t="s">
+        <v>91</v>
+      </c>
+      <c r="B81" s="1">
+        <v>0.05908325448672747</v>
+      </c>
+      <c r="C81" s="1">
+        <v>0.06132067377813355</v>
+      </c>
+      <c r="D81" s="1">
+        <v>0.0378689242974708</v>
+      </c>
+      <c r="E81" s="2">
+        <v>0.01199719871752923</v>
+      </c>
+      <c r="F81" s="2">
+        <v>0.02404588990664133</v>
+      </c>
+      <c r="G81" s="2">
+        <v>0.04770602881179202</v>
+      </c>
+      <c r="H81" s="1">
+        <v>0</v>
+      </c>
+      <c r="I81" s="3">
+        <v>4</v>
+      </c>
+      <c r="J81" t="s">
+        <v>98</v>
+      </c>
+      <c r="K81" s="1">
+        <v>0.3363385925369397</v>
+      </c>
+      <c r="L81" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12">
+      <c r="A82" t="s">
+        <v>92</v>
+      </c>
+      <c r="B82" s="1">
+        <v>0.04717168649752912</v>
+      </c>
+      <c r="C82" s="1">
+        <v>0.03863070895415688</v>
+      </c>
+      <c r="D82" s="1">
+        <v>0.1810615260452819</v>
+      </c>
+      <c r="E82" s="2">
+        <v>0.01956713212067461</v>
+      </c>
+      <c r="F82" s="2">
+        <v>0.02009667190648317</v>
+      </c>
+      <c r="G82" s="2">
+        <v>0.02348382233275986</v>
+      </c>
+      <c r="H82" s="1">
+        <v>0</v>
+      </c>
+      <c r="I82" s="3">
+        <v>2</v>
+      </c>
+      <c r="J82" t="s">
+        <v>99</v>
+      </c>
+      <c r="K82" s="1">
+        <v>0.8682694715752567</v>
+      </c>
+      <c r="L82" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12">
+      <c r="A83" t="s">
+        <v>93</v>
+      </c>
+      <c r="B83" s="1">
+        <v>0.03276772919265269</v>
+      </c>
+      <c r="C83" s="1">
+        <v>0.1154459919352533</v>
+      </c>
+      <c r="D83" s="1">
+        <v>2.523161194860553</v>
+      </c>
+      <c r="E83" s="2">
+        <v>0.005518124626677998</v>
+      </c>
+      <c r="F83" s="2">
+        <v>0.01700548917533124</v>
+      </c>
+      <c r="G83" s="2">
+        <v>0.04896875013194432</v>
+      </c>
+      <c r="H83" s="1">
+        <v>0.4690708740295517</v>
+      </c>
+      <c r="I83" s="3">
+        <v>13</v>
+      </c>
+      <c r="J83">
+        <v>15</v>
+      </c>
+      <c r="K83" s="1">
+        <v>0.9400943396226416</v>
+      </c>
+      <c r="L83" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12">
+      <c r="A84" t="s">
+        <v>94</v>
+      </c>
+      <c r="B84" s="1">
+        <v>0.02830522044005201</v>
+      </c>
+      <c r="C84" s="1">
+        <v>0.000537649784082106</v>
+      </c>
+      <c r="D84" s="1">
+        <v>0.9810052783294586</v>
+      </c>
+      <c r="E84" s="2">
+        <v>0.006813647344864129</v>
+      </c>
+      <c r="F84" s="2">
+        <v>0.002113801669740381</v>
+      </c>
+      <c r="G84" s="2">
+        <v>3.070738238636901E-05</v>
+      </c>
+      <c r="H84" s="1">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3">
+        <v>2</v>
+      </c>
+      <c r="J84" t="s">
+        <v>99</v>
+      </c>
+      <c r="K84" s="1">
+        <v>0.8637615827698473</v>
+      </c>
+      <c r="L84" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12">
+      <c r="A85" t="s">
         <v>95</v>
       </c>
+      <c r="B85" s="1">
+        <v>0.01645162666613142</v>
+      </c>
+      <c r="C85" s="1">
+        <v>0.0607544256012813</v>
+      </c>
+      <c r="D85" s="1">
+        <v>2.692912976584559</v>
+      </c>
+      <c r="E85" s="2">
+        <v>0.002596531029258583</v>
+      </c>
+      <c r="F85" s="2">
+        <v>0.006850898132628285</v>
+      </c>
+      <c r="G85" s="2">
+        <v>0.02357206989954401</v>
+      </c>
+      <c r="H85" s="1">
+        <v>0.02930127723516153</v>
+      </c>
+      <c r="I85" s="3">
+        <v>14</v>
+      </c>
+      <c r="J85">
+        <v>0</v>
+      </c>
+      <c r="K85" s="1">
+        <v>0.8083075335397317</v>
+      </c>
+      <c r="L85" t="s">
+        <v>100</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L78"/>
+  <autoFilter ref="A1:L85"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>